<commit_message>
feat(saison1): tactique, reset hebdo, tickets de tour, notifications privées
- /tactique : égoïste / pragmatique / all-in (cible du sort de soin), figée
  pendant le combat.
- Reset de l'arbre : un par semaine calendaire (lundi 00h, Paris), non
  cumulable.
- Tickets de tour solo : 1/jour + 1 avec la case Confort, non cumulables,
  affichés dans /cd ; consume() prêt pour la future tour.
- Cases Confort : MP quand un temps de recharge est fini (une fois par
  échéance) et MP avec le lien à chaque événement.
- Joueurs : texte lisible des effets (menu Investir, infobulle web), classes
  sur la bannière /profil.
- Garde-fou HARD_MAX_TURNS : un groupe de Soigneurs ne bloque plus un combat.
- Tuto, aide en jeu, CLAUDE.md et tableur à jour.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sakura_content.xlsx
+++ b/docs/sakura_content.xlsx
@@ -27,7 +27,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'📦 Ressources'!$A$1:$H$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'🛠️ Recettes'!$A$1:$G$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'🏪 Shop'!$A$1:$H$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'🌳 Skill Tree'!$A$1:$M$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'🌳 Skill Tree'!$A$1:$M$84</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'🏷️ Titres'!$A$1:$H$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'🌸 Panoplies'!$A$1:$I$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'🐉 World Bosses'!$A$1:$M$6</definedName>
@@ -513,7 +513,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 2026-10-13 21:00 UTC</t>
+          <t>Généré le 2026-10-20 18:20 UTC</t>
         </is>
       </c>
     </row>
@@ -11751,18 +11751,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M43"/>
+  <dimension ref="A1:M84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="48" customWidth="1" min="8" max="8"/>
-    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="39" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
@@ -11905,7 +11905,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Voie de l'Attaque</t>
+          <t>Voie du Guerrier</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11915,7 +11915,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Stats</t>
+          <t>Voies</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
@@ -11929,7 +11929,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>atk_percent → [5]</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -11948,11 +11948,7 @@
           <t>⚔️</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Début de voie — à étoffer.</t>
-        </is>
-      </c>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -11962,7 +11958,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Voie de la Défense</t>
+          <t>Voie du Protecteur</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -11972,7 +11968,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Stats</t>
+          <t>Voies</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr"/>
@@ -11986,7 +11982,7 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>def_percent → [5]</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
@@ -12005,11 +12001,7 @@
           <t>🛡️</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
-        <is>
-          <t>Début de voie — à étoffer.</t>
-        </is>
-      </c>
+      <c r="M4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -12029,7 +12021,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Stats</t>
+          <t>Voies</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
@@ -12043,7 +12035,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>hp_max_percent → [5]</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -12062,11 +12054,7 @@
           <t>❤️</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Début de voie — à étoffer.</t>
-        </is>
-      </c>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -12086,7 +12074,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Classe</t>
+          <t>Classes</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr"/>
@@ -12098,14 +12086,16 @@
           <t>1</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>grant_class → [combattant]
+hp_max_percent → [5]
+atk_percent → [5]</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Attaque, Défense, Défense, Attaque</t>
+          <t>Attaque, Deg. Crit., Défense, Régénération</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
@@ -12120,12 +12110,12 @@
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>🦾</t>
+          <t>👊</t>
         </is>
       </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>Classe obtenue en reliant deux voies.</t>
+          <t>Classe Combattant : +5 % de PV max et +5 % d'attaque.</t>
         </is>
       </c>
     </row>
@@ -12147,7 +12137,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Classe</t>
+          <t>Classes</t>
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
@@ -12159,14 +12149,16 @@
           <t>1</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>grant_class → [paladin]
+heal_received_percent → [50]
+def_percent → [5]</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Support, Défense, Support, Défense</t>
+          <t>PV, Défense, Régénération, Rég. Mana</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -12186,7 +12178,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Classe obtenue en reliant deux voies.</t>
+          <t>Classe Paladin : soins reçus +50 % et +5 % de défense.</t>
         </is>
       </c>
     </row>
@@ -12208,7 +12200,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Classe</t>
+          <t>Classes</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr"/>
@@ -12220,14 +12212,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>grant_class → [vampire]
+lifesteal_percent → [5]</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>Attaque, Support, Attaque, Support</t>
+          <t>Attaque, Deg. Crit., PV, Rég. Mana</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
@@ -12242,12 +12235,12 @@
       </c>
       <c r="L8" s="5" t="inlineStr">
         <is>
-          <t>🩸</t>
+          <t>🧛</t>
         </is>
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>Classe obtenue en reliant deux voies.</t>
+          <t>Classe Vampire : se soigne de 5 % des dégâts infligés.</t>
         </is>
       </c>
     </row>
@@ -12298,7 +12291,7 @@
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>1820, 500</t>
+          <t>1090, -230</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -12320,7 +12313,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Axe de l'Or</t>
+          <t>Bonus Or</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -12330,7 +12323,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Stats</t>
+          <t>Passives</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr"/>
@@ -12344,7 +12337,7 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>gold_drop_percent → [1,3,5]</t>
+          <t>gold_drop_percent → [1,4,10]</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
@@ -12355,7 +12348,7 @@
       <c r="J10" s="5" t="inlineStr"/>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>1954, 634</t>
+          <t>1224, -96</t>
         </is>
       </c>
       <c r="L10" s="5" t="inlineStr">
@@ -12363,11 +12356,7 @@
           <t>💰</t>
         </is>
       </c>
-      <c r="M10" s="5" t="inlineStr">
-        <is>
-          <t>Début d'axe — à étoffer.</t>
-        </is>
-      </c>
+      <c r="M10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -12377,7 +12366,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Axe du Butin</t>
+          <t>Chance Drop</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -12387,7 +12376,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Stats</t>
+          <t>Passives</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
@@ -12401,12 +12390,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>drop_rate_multiplier → [1,3,5]</t>
+          <t>drop_rate_multiplier → [10,40,100]</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Axe de l'Or, Axe de l'Expérience</t>
+          <t>Bonus Or, Bonus XP</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -12416,7 +12405,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>1820, 785</t>
+          <t>1090, 55</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -12424,11 +12413,7 @@
           <t>🍀</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>Début d'axe — à étoffer.</t>
-        </is>
-      </c>
+      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -12438,7 +12423,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Axe de l'Expérience</t>
+          <t>Bonus XP</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -12448,7 +12433,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Stats</t>
+          <t>Passives</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr"/>
@@ -12462,7 +12447,7 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>xp_drop_percent → [1,3,5]</t>
+          <t>xp_drop_percent → [1,4,10]</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
@@ -12473,7 +12458,7 @@
       <c r="J12" s="5" t="inlineStr"/>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>1686, 634</t>
+          <t>956, -96</t>
         </is>
       </c>
       <c r="L12" s="5" t="inlineStr">
@@ -12481,11 +12466,7 @@
           <t>⚡</t>
         </is>
       </c>
-      <c r="M12" s="5" t="inlineStr">
-        <is>
-          <t>Début d'axe — à étoffer.</t>
-        </is>
-      </c>
+      <c r="M12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -12495,7 +12476,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Axe du Confort</t>
+          <t>Confort</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -12505,34 +12486,32 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Stats</t>
+          <t>Passives</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>1,2,3</t>
-        </is>
-      </c>
-      <c r="H13" s="8" t="inlineStr">
-        <is>
-          <t>unlock_feature → [Notification privé lorsque le cooldown d'une commande est prêt,Notification privé lorsque le cooldown d'une commande est prêt,Notification privé lorsque le cooldown d'une commande est prêt]
-unlock_feature → [1 participation journalière supplémentaire pour défier la tour solo,1 participation journalière supplémentaire pour défier la tour solo,1 participation journalière supplémentaire pour défier la tour solo]
-unlock_feature → [Notifié lorsqu'un événement aparait,Notifié lorsqu'un événement aparait,Notifié lorsqu'un événement aparait]</t>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>unlock_feature → [notify_cooldowns]</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Axe du Butin</t>
+          <t>Chance Drop</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>1820, 975</t>
+          <t>1090, 245</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -12542,7 +12521,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Début d'axe — à étoffer.</t>
+          <t>Reçois un message privé quand un de tes temps de recharge est terminé.</t>
         </is>
       </c>
     </row>
@@ -12554,17 +12533,17 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
           <t>Support</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Support</t>
-        </is>
-      </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr"/>
@@ -12578,7 +12557,7 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>hp_max_percent → [1]</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
@@ -12602,22 +12581,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>passif_3</t>
+          <t>passif_4</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>Vitesse</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
           <t>Support</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Support</t>
-        </is>
-      </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats Avancées</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
@@ -12631,23 +12610,23 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>speed_flat → [1]</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Support</t>
+          <t>PV</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>-574, 735</t>
+          <t>-416, 786</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>💧</t>
+          <t>💨</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -12655,22 +12634,22 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>passif_4</t>
+          <t>passif_5</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
+          <t>Vitesse</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
           <t>Support</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Support</t>
-        </is>
-      </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats Avancées</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr"/>
@@ -12684,18 +12663,18 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>speed_flat → [1]</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>Support</t>
+          <t>PV</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr"/>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t>-416, 786</t>
+          <t>-539, 573</t>
         </is>
       </c>
       <c r="L16" s="5" t="inlineStr">
@@ -12708,22 +12687,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>passif_5</t>
+          <t>passif_6</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
           <t>Support</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Support</t>
-        </is>
-      </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
@@ -12737,23 +12716,23 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>hp_max_percent → [1]</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Support</t>
+          <t>Vitesse</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>-539, 573</t>
+          <t>-650, 450</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>💨</t>
+          <t>❤️</t>
         </is>
       </c>
       <c r="M17" t="inlineStr"/>
@@ -12761,22 +12740,22 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>passif_6</t>
+          <t>passif_7</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
           <t>Support</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Support</t>
-        </is>
-      </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr"/>
@@ -12790,22 +12769,18 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>hp_max_percent → [1]</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>Support, Support</t>
-        </is>
-      </c>
-      <c r="J18" s="5" t="inlineStr">
-        <is>
-          <t>toutes</t>
-        </is>
-      </c>
+          <t>Vitesse</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr"/>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t>-650, 450</t>
+          <t>-366, 943</t>
         </is>
       </c>
       <c r="L18" s="5" t="inlineStr">
@@ -12818,22 +12793,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>passif_7</t>
+          <t>passif_8</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
           <t>Support</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Support</t>
-        </is>
-      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
@@ -12847,22 +12822,18 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>hp_max_percent → [1]</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Support, Support</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>toutes</t>
-        </is>
-      </c>
+          <t>Voie du Support</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-366, 943</t>
+          <t>-222, 697</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -12875,22 +12846,22 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>passif_8</t>
+          <t>passif_9</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
           <t>Support</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Support</t>
-        </is>
-      </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr"/>
@@ -12904,18 +12875,18 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>hp_max_percent → [1]</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>Support</t>
+          <t>Voie du Support</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr"/>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t>-222, 697</t>
+          <t>-365, 450</t>
         </is>
       </c>
       <c r="L20" s="5" t="inlineStr">
@@ -12928,22 +12899,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>passif_9</t>
+          <t>stat_1</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Support</t>
+          <t>Défense</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Support</t>
+          <t>Défense</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
@@ -12957,23 +12928,23 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>def_percent → [1]</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Support</t>
+          <t>Voie du Protecteur</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-365, 450</t>
+          <t>249, 640</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>❤️</t>
+          <t>🛡️</t>
         </is>
       </c>
       <c r="M21" t="inlineStr"/>
@@ -12981,22 +12952,22 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>stat_1</t>
+          <t>actif_1</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Défense</t>
+          <t>Attaque</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Défense</t>
+          <t>Attaque</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr"/>
@@ -13010,23 +12981,23 @@
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>atk_percent → [1]</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>Voie de la Défense</t>
+          <t>Voie du Guerrier</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr"/>
       <c r="K22" s="5" t="inlineStr">
         <is>
-          <t>249, 640</t>
+          <t>-80, 70</t>
         </is>
       </c>
       <c r="L22" s="5" t="inlineStr">
         <is>
-          <t>🛡️</t>
+          <t>⚔️</t>
         </is>
       </c>
       <c r="M22" s="5" t="inlineStr"/>
@@ -13034,7 +13005,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>actif_1</t>
+          <t>actif_2</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -13049,7 +13020,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats</t>
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
@@ -13063,18 +13034,18 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>atk_percent → [1]</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Voie de l'Attaque</t>
+          <t>Voie du Guerrier</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
-          <t>-80, 70</t>
+          <t>-222, 203</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -13087,7 +13058,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>actif_2</t>
+          <t>actif_3</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -13102,7 +13073,7 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr"/>
@@ -13116,18 +13087,18 @@
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>atk_percent → [1]</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>Attaque</t>
+          <t>Voie du Guerrier</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr"/>
       <c r="K24" s="5" t="inlineStr">
         <is>
-          <t>-222, 203</t>
+          <t>63, 203</t>
         </is>
       </c>
       <c r="L24" s="5" t="inlineStr">
@@ -13140,22 +13111,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>actif_3</t>
+          <t>actif_6</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>Vitesse</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Attaque</t>
-        </is>
-      </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats Avancées</t>
         </is>
       </c>
       <c r="E25" t="inlineStr"/>
@@ -13169,7 +13140,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>speed_flat → [1]</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -13180,12 +13151,12 @@
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
-          <t>63, 203</t>
+          <t>-203, -9</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>⚔️</t>
+          <t>💨</t>
         </is>
       </c>
       <c r="M25" t="inlineStr"/>
@@ -13193,7 +13164,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>actif_5</t>
+          <t>actif_7</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
@@ -13208,7 +13179,7 @@
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr"/>
@@ -13222,23 +13193,23 @@
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>atk_percent → [1]</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t>Attaque</t>
+          <t>Vitesse</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr"/>
       <c r="K26" s="5" t="inlineStr">
         <is>
-          <t>-80, -120</t>
+          <t>-365, -44</t>
         </is>
       </c>
       <c r="L26" s="5" t="inlineStr">
         <is>
-          <t>🎯</t>
+          <t>⚔️</t>
         </is>
       </c>
       <c r="M26" s="5" t="inlineStr"/>
@@ -13246,22 +13217,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>actif_6</t>
+          <t>actif_8</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
+          <t>Vitesse</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Attaque</t>
-        </is>
-      </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats Avancées</t>
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
@@ -13275,7 +13246,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>speed_flat → [1]</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -13286,7 +13257,7 @@
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>-203, -9</t>
+          <t>43, -9</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -13299,7 +13270,7 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>actif_7</t>
+          <t>actif_9</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
@@ -13314,7 +13285,7 @@
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr"/>
@@ -13328,22 +13299,18 @@
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>atk_percent → [1]</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>Attaque, Attaque</t>
-        </is>
-      </c>
-      <c r="J28" s="5" t="inlineStr">
-        <is>
-          <t>toutes</t>
-        </is>
-      </c>
+          <t>Vitesse</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr"/>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t>-365, -44</t>
+          <t>205, -44</t>
         </is>
       </c>
       <c r="L28" s="5" t="inlineStr">
@@ -13356,22 +13323,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>actif_8</t>
+          <t>actif_10</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t>Deg. Crit.</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Attaque</t>
-        </is>
-      </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats Avancées</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
@@ -13385,7 +13352,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>crit_damage_flat → [5]</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -13396,12 +13363,12 @@
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
-          <t>43, -9</t>
+          <t>-416, 114</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>💨</t>
+          <t>💥</t>
         </is>
       </c>
       <c r="M29" t="inlineStr"/>
@@ -13409,22 +13376,22 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>actif_9</t>
+          <t>actif_11</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
+          <t>Deg. Crit.</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>Attaque</t>
-        </is>
-      </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats Avancées</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr"/>
@@ -13438,27 +13405,23 @@
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>crit_damage_flat → [5]</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t>Attaque, Attaque</t>
-        </is>
-      </c>
-      <c r="J30" s="5" t="inlineStr">
-        <is>
-          <t>toutes</t>
-        </is>
-      </c>
+          <t>Attaque</t>
+        </is>
+      </c>
+      <c r="J30" s="5" t="inlineStr"/>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t>205, -44</t>
+          <t>256, 114</t>
         </is>
       </c>
       <c r="L30" s="5" t="inlineStr">
         <is>
-          <t>⚔️</t>
+          <t>💥</t>
         </is>
       </c>
       <c r="M30" s="5" t="inlineStr"/>
@@ -13466,22 +13429,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>actif_10</t>
+          <t>stat_3</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Attaque</t>
+          <t>Défense</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Attaque</t>
+          <t>Défense</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
@@ -13495,23 +13458,23 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>def_percent → [1]</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Attaque</t>
+          <t>Voie du Protecteur</t>
         </is>
       </c>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr">
         <is>
-          <t>-416, 114</t>
+          <t>63, 697</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>💥</t>
+          <t>🛡️</t>
         </is>
       </c>
       <c r="M31" t="inlineStr"/>
@@ -13519,22 +13482,22 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>actif_11</t>
+          <t>stat_4</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Attaque</t>
+          <t>Défense</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Attaque</t>
+          <t>Défense</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr"/>
@@ -13548,23 +13511,23 @@
       </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>def_percent → [1]</t>
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>Attaque</t>
+          <t>Voie du Protecteur</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr"/>
       <c r="K32" s="5" t="inlineStr">
         <is>
-          <t>256, 114</t>
+          <t>205, 450</t>
         </is>
       </c>
       <c r="L32" s="5" t="inlineStr">
         <is>
-          <t>💥</t>
+          <t>🛡️</t>
         </is>
       </c>
       <c r="M32" s="5" t="inlineStr"/>
@@ -13572,22 +13535,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>stat_3</t>
+          <t>stat_7</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
+          <t>Vitesse</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
           <t>Défense</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Défense</t>
-        </is>
-      </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats Avancées</t>
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
@@ -13601,7 +13564,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>speed_flat → [1]</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -13612,12 +13575,12 @@
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr">
         <is>
-          <t>63, 697</t>
+          <t>379, 573</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>🛡️</t>
+          <t>💨</t>
         </is>
       </c>
       <c r="M33" t="inlineStr"/>
@@ -13625,7 +13588,7 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>stat_4</t>
+          <t>stat_8</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
@@ -13640,7 +13603,7 @@
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr"/>
@@ -13654,18 +13617,18 @@
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>def_percent → [1]</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
-          <t>Défense</t>
+          <t>Vitesse</t>
         </is>
       </c>
       <c r="J34" s="5" t="inlineStr"/>
       <c r="K34" s="5" t="inlineStr">
         <is>
-          <t>205, 450</t>
+          <t>490, 450</t>
         </is>
       </c>
       <c r="L34" s="5" t="inlineStr">
@@ -13678,22 +13641,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>stat_5</t>
+          <t>stat_9</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
+          <t>Vitesse</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
           <t>Défense</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Défense</t>
-        </is>
-      </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats Avancées</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
@@ -13707,7 +13670,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>speed_flat → [1]</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -13718,12 +13681,12 @@
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
-          <t>414, 735</t>
+          <t>256, 786</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>🌀</t>
+          <t>💨</t>
         </is>
       </c>
       <c r="M35" t="inlineStr"/>
@@ -13731,22 +13694,22 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>stat_7</t>
+          <t>stat_10</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
+          <t>Régénération</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
           <t>Défense</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>Défense</t>
-        </is>
-      </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats Avancées</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr"/>
@@ -13760,7 +13723,7 @@
       </c>
       <c r="H36" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>hp_regeneration_flat → [5]</t>
         </is>
       </c>
       <c r="I36" s="5" t="inlineStr">
@@ -13771,12 +13734,12 @@
       <c r="J36" s="5" t="inlineStr"/>
       <c r="K36" s="5" t="inlineStr">
         <is>
-          <t>379, 573</t>
+          <t>43, 909</t>
         </is>
       </c>
       <c r="L36" s="5" t="inlineStr">
         <is>
-          <t>💨</t>
+          <t>✨</t>
         </is>
       </c>
       <c r="M36" s="5" t="inlineStr"/>
@@ -13784,22 +13747,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>stat_8</t>
+          <t>stat_2</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
+          <t>Régénération</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
           <t>Défense</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Défense</t>
-        </is>
-      </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats Avancées</t>
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
@@ -13813,27 +13776,23 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>hp_regeneration_flat → [5]</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Défense, Défense</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>toutes</t>
-        </is>
-      </c>
+          <t>Défense</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
-          <t>490, 450</t>
+          <t>379, 327</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>🛡️</t>
+          <t>✨</t>
         </is>
       </c>
       <c r="M37" t="inlineStr"/>
@@ -13841,7 +13800,7 @@
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>stat_9</t>
+          <t>stat_6</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
@@ -13856,7 +13815,7 @@
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr"/>
@@ -13870,23 +13829,23 @@
       </c>
       <c r="H38" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>def_percent → [1]</t>
         </is>
       </c>
       <c r="I38" s="5" t="inlineStr">
         <is>
-          <t>Défense</t>
+          <t>Vitesse</t>
         </is>
       </c>
       <c r="J38" s="5" t="inlineStr"/>
       <c r="K38" s="5" t="inlineStr">
         <is>
-          <t>256, 786</t>
+          <t>205, 944</t>
         </is>
       </c>
       <c r="L38" s="5" t="inlineStr">
         <is>
-          <t>💨</t>
+          <t>🛡️</t>
         </is>
       </c>
       <c r="M38" s="5" t="inlineStr"/>
@@ -13894,22 +13853,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>stat_10</t>
+          <t>passif_2</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Défense</t>
+          <t>Rég. Mana</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Défense</t>
+          <t>Support</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats Avancées</t>
         </is>
       </c>
       <c r="E39" t="inlineStr"/>
@@ -13923,23 +13882,23 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>mana_regeneration_flat → [1]</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Défense</t>
+          <t>PV</t>
         </is>
       </c>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr">
         <is>
-          <t>43, 909</t>
+          <t>-204, 909</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>✨</t>
+          <t>🔷</t>
         </is>
       </c>
       <c r="M39" t="inlineStr"/>
@@ -13947,22 +13906,22 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>stat_2</t>
+          <t>passif_10</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Défense</t>
+          <t>Rég. Mana</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Défense</t>
+          <t>Support</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats Avancées</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr"/>
@@ -13976,23 +13935,23 @@
       </c>
       <c r="H40" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>mana_regeneration_flat → [1]</t>
         </is>
       </c>
       <c r="I40" s="5" t="inlineStr">
         <is>
-          <t>Défense</t>
+          <t>PV</t>
         </is>
       </c>
       <c r="J40" s="5" t="inlineStr"/>
       <c r="K40" s="5" t="inlineStr">
         <is>
-          <t>379, 327</t>
+          <t>-539, 327</t>
         </is>
       </c>
       <c r="L40" s="5" t="inlineStr">
         <is>
-          <t>✨</t>
+          <t>🔷</t>
         </is>
       </c>
       <c r="M40" s="5" t="inlineStr"/>
@@ -14000,22 +13959,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>stat_6</t>
+          <t>passif_14</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Défense</t>
+          <t>AOE</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Défense</t>
+          <t>Mage</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Passives</t>
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
@@ -14029,12 +13988,12 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>splash_damage_percent → [25]</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Défense, Défense</t>
+          <t>Rég. Mana, Deg. Crit.</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -14044,35 +14003,39 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>205, 944</t>
+          <t>-574, 165</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>🛡️</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr"/>
+          <t>🔮</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Les attaques infligent aussi des dégats aux ennemis adjacents la cible, 25% de dégats de l'attaque.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>passif_2</t>
+          <t>type_1_6</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Support</t>
+          <t>Mage</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>Support</t>
+          <t>Classe</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Classes</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr"/>
@@ -14084,48 +14047,57 @@
           <t>1</t>
         </is>
       </c>
-      <c r="H42" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>grant_class → [mage]
+mage_affinity_bonus → [1]</t>
         </is>
       </c>
       <c r="I42" s="5" t="inlineStr">
         <is>
-          <t>Support</t>
-        </is>
-      </c>
-      <c r="J42" s="5" t="inlineStr"/>
+          <t>Deg. Crit., Rég. Mana</t>
+        </is>
+      </c>
+      <c r="J42" s="5" t="inlineStr">
+        <is>
+          <t>toutes</t>
+        </is>
+      </c>
       <c r="K42" s="5" t="inlineStr">
         <is>
-          <t>-204, 909</t>
+          <t>-820, 22</t>
         </is>
       </c>
       <c r="L42" s="5" t="inlineStr">
         <is>
-          <t>🔷</t>
-        </is>
-      </c>
-      <c r="M42" s="5" t="inlineStr"/>
+          <t>🧙</t>
+        </is>
+      </c>
+      <c r="M42" s="5" t="inlineStr">
+        <is>
+          <t>Classe Mage : dégâts ×1,5 si son affinité dans l'élément de l'attaque atteint 25, ×2 à 50, ×5 à 100.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>passif_10</t>
+          <t>type_1_8</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Support</t>
+          <t>Chance Crit.</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Support</t>
+          <t>Mage</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Départ</t>
+          <t>Stats Avancées</t>
         </is>
       </c>
       <c r="E43" t="inlineStr"/>
@@ -14139,29 +14111,2307 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>crit_chance_flat → [1]</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Support</t>
+          <t>AOE</t>
         </is>
       </c>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr">
         <is>
-          <t>-539, 327</t>
+          <t>-550, -20</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
+          <t>🎯</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>type_1_10</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Mana</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Mage</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Stats Avancées</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr"/>
+      <c r="F44" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
+          <t>mana_max_flat → [5]</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="inlineStr">
+        <is>
+          <t>AOE</t>
+        </is>
+      </c>
+      <c r="J44" s="5" t="inlineStr"/>
+      <c r="K44" s="5" t="inlineStr">
+        <is>
+          <t>-722, 278</t>
+        </is>
+      </c>
+      <c r="L44" s="5" t="inlineStr">
+        <is>
+          <t>💧</t>
+        </is>
+      </c>
+      <c r="M44" s="5" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>type_1_1</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Rég. Mana</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Mage</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Stats Avancées</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>mana_regeneration_flat → [1]</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Mana</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>-906, 229</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
           <t>🔷</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>type_1_2</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Deg. Crit.</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Mage</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Stats Avancées</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr"/>
+      <c r="F46" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>crit_damage_flat → [5]</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr">
+        <is>
+          <t>Chance Crit.</t>
+        </is>
+      </c>
+      <c r="J46" s="5" t="inlineStr"/>
+      <c r="K46" s="5" t="inlineStr">
+        <is>
+          <t>-685, -155</t>
+        </is>
+      </c>
+      <c r="L46" s="5" t="inlineStr">
+        <is>
+          <t>💥</t>
+        </is>
+      </c>
+      <c r="M46" s="5" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>passif_11</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Résistant</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Passives</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>damage_taken_reduction_percent → [10]</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Rég. Mana, Régénération</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>toutes</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>-80, 1020</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>🫧</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>Réduit de 10% les dégats reçus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>type_1_3</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Egide</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Classe</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Classes</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr"/>
+      <c r="F48" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>grant_class → [egide]
+team_shield_percent → [10]</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>Rég. Mana, Régénération</t>
+        </is>
+      </c>
+      <c r="J48" s="5" t="inlineStr">
+        <is>
+          <t>toutes</t>
+        </is>
+      </c>
+      <c r="K48" s="5" t="inlineStr">
+        <is>
+          <t>-80, 1305</t>
+        </is>
+      </c>
+      <c r="L48" s="5" t="inlineStr">
+        <is>
+          <t>🗿</t>
+        </is>
+      </c>
+      <c r="M48" s="5" t="inlineStr">
+        <is>
+          <t>Au début du combat donne un bouclier de 10% de ses points de vie max à lui et tous ses alliés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>type_1_4</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Mana</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Stats Avancées</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>mana_max_flat → [5]</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Résistant</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>-252, 1092</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>💧</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>type_1_5</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Esquive</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Stats Avancées</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr"/>
+      <c r="F50" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
+          <t>dodge_flat → [1]</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>Résistant</t>
+        </is>
+      </c>
+      <c r="J50" s="5" t="inlineStr"/>
+      <c r="K50" s="5" t="inlineStr">
+        <is>
+          <t>92, 1092</t>
+        </is>
+      </c>
+      <c r="L50" s="5" t="inlineStr">
+        <is>
+          <t>🌀</t>
+        </is>
+      </c>
+      <c r="M50" s="5" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>type_1_7</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Régénération</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Stats Avancées</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>hp_regeneration_flat → [5]</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Esquive</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>141, 1276</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>✨</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>type_1_9</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Rég. Mana</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Stats Avancées</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr"/>
+      <c r="F52" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>mana_regeneration_flat → [1]</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>Mana</t>
+        </is>
+      </c>
+      <c r="J52" s="5" t="inlineStr"/>
+      <c r="K52" s="5" t="inlineStr">
+        <is>
+          <t>-301, 1276</t>
+        </is>
+      </c>
+      <c r="L52" s="5" t="inlineStr">
+        <is>
+          <t>🔷</t>
+        </is>
+      </c>
+      <c r="M52" s="5" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>passif_12</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Tenace</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Sentinelle</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Passives</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>last_stand → [1]</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Deg. Crit., Régénération</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>toutes</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>414, 165</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>💀</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>Lors d'un combat, la première attaque devant le tuer le laisse à 1 pv à la place.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>type_1_11</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Titan</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>Classe</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Classes</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr"/>
+      <c r="F54" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H54" s="7" t="inlineStr">
+        <is>
+          <t>grant_class → [titan]
+damage_dealt_percent → [5]
+damage_taken_reduction_percent → [5]</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>Deg. Crit., Régénération</t>
+        </is>
+      </c>
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>toutes</t>
+        </is>
+      </c>
+      <c r="K54" s="5" t="inlineStr">
+        <is>
+          <t>660, 23</t>
+        </is>
+      </c>
+      <c r="L54" s="5" t="inlineStr">
+        <is>
+          <t>🦾</t>
+        </is>
+      </c>
+      <c r="M54" s="5" t="inlineStr">
+        <is>
+          <t>Inflige 5% de dégats supplémentaires et réduit de 5% les dégats reçus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>type_1_12</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Chance Crit.</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Sentinelle</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Stats Avancées</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>crit_chance_flat → [1]</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Tenace</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>390, -20</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>🎯</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>type_1_13</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Esquive</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Sentinelle</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Stats Avancées</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr"/>
+      <c r="F56" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H56" s="5" t="inlineStr">
+        <is>
+          <t>dodge_flat → [1]</t>
+        </is>
+      </c>
+      <c r="I56" s="5" t="inlineStr">
+        <is>
+          <t>Tenace</t>
+        </is>
+      </c>
+      <c r="J56" s="5" t="inlineStr"/>
+      <c r="K56" s="5" t="inlineStr">
+        <is>
+          <t>562, 278</t>
+        </is>
+      </c>
+      <c r="L56" s="5" t="inlineStr">
+        <is>
+          <t>🌀</t>
+        </is>
+      </c>
+      <c r="M56" s="5" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>type_1_14</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Régénération</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Sentinelle</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Stats Avancées</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>hp_regeneration_flat → [5]</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Esquive</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>746, 229</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>✨</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>type_1_15</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Deg. Crit.</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>Sentinelle</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Stats Avancées</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr"/>
+      <c r="F58" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H58" s="5" t="inlineStr">
+        <is>
+          <t>crit_damage_flat → [5]</t>
+        </is>
+      </c>
+      <c r="I58" s="5" t="inlineStr">
+        <is>
+          <t>Chance Crit.</t>
+        </is>
+      </c>
+      <c r="J58" s="5" t="inlineStr"/>
+      <c r="K58" s="5" t="inlineStr">
+        <is>
+          <t>525, -155</t>
+        </is>
+      </c>
+      <c r="L58" s="5" t="inlineStr">
+        <is>
+          <t>💥</t>
+        </is>
+      </c>
+      <c r="M58" s="5" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>passif_13</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Mana</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Stats Avancées</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>mana_max_flat → [5]</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>-935, 450</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>💧</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>passif_15</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>Mana</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Stats Avancées</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr"/>
+      <c r="F60" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H60" s="5" t="inlineStr">
+        <is>
+          <t>mana_max_flat → [5]</t>
+        </is>
+      </c>
+      <c r="I60" s="5" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="J60" s="5" t="inlineStr"/>
+      <c r="K60" s="5" t="inlineStr">
+        <is>
+          <t>-507, 1190</t>
+        </is>
+      </c>
+      <c r="L60" s="5" t="inlineStr">
+        <is>
+          <t>💧</t>
+        </is>
+      </c>
+      <c r="M60" s="5" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>passif_16</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Soigneur</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Classe</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Classes</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H61" s="8" t="inlineStr">
+        <is>
+          <t>grant_class → [soigneur]
+healer_spell → [1]
+heal_power_multiplier → [2]
+speed_per_ally → [1]</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Rég. Mana, Rég. Mana</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>toutes</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>-820, 878</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>💚</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>Classe Soigneur : remplace son attaque par un sort de soin (cible choisie selon sa tactique, /tactique), soins donnés doublés, +1 de vitesse par allié présent au combat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>passif_17</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>Rég. Mana</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Stats Avancées</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr"/>
+      <c r="F62" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G62" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H62" s="5" t="inlineStr">
+        <is>
+          <t>mana_regeneration_flat → [1]</t>
+        </is>
+      </c>
+      <c r="I62" s="5" t="inlineStr">
+        <is>
+          <t>Mana</t>
+        </is>
+      </c>
+      <c r="J62" s="5" t="inlineStr"/>
+      <c r="K62" s="5" t="inlineStr">
+        <is>
+          <t>-906, 671</t>
+        </is>
+      </c>
+      <c r="L62" s="5" t="inlineStr">
+        <is>
+          <t>🔷</t>
+        </is>
+      </c>
+      <c r="M62" s="5" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>passif_18</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Rég. Mana</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Stats Avancées</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>mana_regeneration_flat → [1]</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Mana</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>-685, 1055</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>🔷</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>passif_3</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>Esquive</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>Défense</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>Stats Avancées</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr"/>
+      <c r="F64" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H64" s="5" t="inlineStr">
+        <is>
+          <t>dodge_flat → [1]</t>
+        </is>
+      </c>
+      <c r="I64" s="5" t="inlineStr">
+        <is>
+          <t>Défense</t>
+        </is>
+      </c>
+      <c r="J64" s="5" t="inlineStr"/>
+      <c r="K64" s="5" t="inlineStr">
+        <is>
+          <t>348, 1190</t>
+        </is>
+      </c>
+      <c r="L64" s="5" t="inlineStr">
+        <is>
+          <t>🌀</t>
+        </is>
+      </c>
+      <c r="M64" s="5" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>passif_19</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Esquive</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Défense</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Stats Avancées</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="n">
+        <v>1</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>dodge_flat → [1]</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Défense</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>775, 450</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>🌀</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>passif_20</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>Rempart</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>Classe</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>Classes</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr"/>
+      <c r="F66" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H66" s="7" t="inlineStr">
+        <is>
+          <t>grant_class → [rempart]
+redirect_ally_damage_percent → [50]</t>
+        </is>
+      </c>
+      <c r="I66" s="5" t="inlineStr">
+        <is>
+          <t>Régénération, Régénération</t>
+        </is>
+      </c>
+      <c r="J66" s="5" t="inlineStr">
+        <is>
+          <t>toutes</t>
+        </is>
+      </c>
+      <c r="K66" s="5" t="inlineStr">
+        <is>
+          <t>660, 878</t>
+        </is>
+      </c>
+      <c r="L66" s="5" t="inlineStr">
+        <is>
+          <t>🧱</t>
+        </is>
+      </c>
+      <c r="M66" s="5" t="inlineStr">
+        <is>
+          <t>Redirige 50% des dégats que devrait recevoir ses alliés sur lui à la place.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>passif_21</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Régénération</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Défense</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Stats Avancées</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="n">
+        <v>1</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>hp_regeneration_flat → [5]</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Esquive</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>525, 1055</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>✨</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>passif_22</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>Régénération</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>Défense</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>Stats Avancées</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr"/>
+      <c r="F68" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H68" s="5" t="inlineStr">
+        <is>
+          <t>hp_regeneration_flat → [5]</t>
+        </is>
+      </c>
+      <c r="I68" s="5" t="inlineStr">
+        <is>
+          <t>Esquive</t>
+        </is>
+      </c>
+      <c r="J68" s="5" t="inlineStr"/>
+      <c r="K68" s="5" t="inlineStr">
+        <is>
+          <t>746, 671</t>
+        </is>
+      </c>
+      <c r="L68" s="5" t="inlineStr">
+        <is>
+          <t>✨</t>
+        </is>
+      </c>
+      <c r="M68" s="5" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>passif_23</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Chance Crit.</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Attaque</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Stats Avancées</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="n">
+        <v>1</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>crit_chance_flat → [1]</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Attaque</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>348, -290</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>🎯</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>passif_24</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>Deg. Crit.</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>Attaque</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>Stats Avancées</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr"/>
+      <c r="F70" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G70" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H70" s="5" t="inlineStr">
+        <is>
+          <t>crit_damage_flat → [5]</t>
+        </is>
+      </c>
+      <c r="I70" s="5" t="inlineStr">
+        <is>
+          <t>Chance Crit.</t>
+        </is>
+      </c>
+      <c r="J70" s="5" t="inlineStr"/>
+      <c r="K70" s="5" t="inlineStr">
+        <is>
+          <t>141, -376</t>
+        </is>
+      </c>
+      <c r="L70" s="5" t="inlineStr">
+        <is>
+          <t>💥</t>
+        </is>
+      </c>
+      <c r="M70" s="5" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>passif_25</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Classe</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Classes</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H71" s="8" t="inlineStr">
+        <is>
+          <t>grant_class → [assassin]
+crit_chance_multiplier → [2]
+crit_damage_multiplier → [3]</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Deg. Crit., Deg. Crit.</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>toutes</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>-80, -405</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>🥷</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>Double ses chances de critique et triple ses dégats critiques.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>passif_26</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>Deg. Crit.</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>Attaque</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>Stats Avancées</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr"/>
+      <c r="F72" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H72" s="5" t="inlineStr">
+        <is>
+          <t>crit_damage_flat → [5]</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>Chance Crit.</t>
+        </is>
+      </c>
+      <c r="J72" s="5" t="inlineStr"/>
+      <c r="K72" s="5" t="inlineStr">
+        <is>
+          <t>-301, -376</t>
+        </is>
+      </c>
+      <c r="L72" s="5" t="inlineStr">
+        <is>
+          <t>💥</t>
+        </is>
+      </c>
+      <c r="M72" s="5" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>passif_27</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Chance Crit.</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Attaque</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Stats Avancées</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="n">
+        <v>1</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>crit_chance_flat → [1]</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Attaque</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>-507, -290</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>🎯</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>passif_28</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>Vaillant</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>Défense</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>Passives</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr"/>
+      <c r="F74" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H74" s="5" t="inlineStr">
+        <is>
+          <t>taunt_chance_percent → [50]</t>
+        </is>
+      </c>
+      <c r="I74" s="5" t="inlineStr">
+        <is>
+          <t>Vitesse, Vitesse</t>
+        </is>
+      </c>
+      <c r="J74" s="5" t="inlineStr">
+        <is>
+          <t>toutes</t>
+        </is>
+      </c>
+      <c r="K74" s="5" t="inlineStr">
+        <is>
+          <t>414, 735</t>
+        </is>
+      </c>
+      <c r="L74" s="5" t="inlineStr">
+        <is>
+          <t>🫀</t>
+        </is>
+      </c>
+      <c r="M74" s="5" t="inlineStr">
+        <is>
+          <t>Durant le combat à 50% de chance d'appliquer provocation sur l'ennemi, la prochaine attaque de l'ennemi devra cibler en priorité le lanceur de provocation, si plusieurs joueurs on lancé provocation, seul le dernier lanceur sera ciblé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>passif_29</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Passives</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="n">
+        <v>1</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>heal_buff_percent → [10]</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Vitesse, Vitesse</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>toutes</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>-574, 735</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>💊</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>Les soins accordent également un bonus pour le combat de 10% d'attaque et 10% de défense sur la cible du soin et sur soit même, non cumulable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t>actif_4</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>Léthal</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>Attaque</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr">
+        <is>
+          <t>Passives</t>
+        </is>
+      </c>
+      <c r="E76" s="5" t="inlineStr"/>
+      <c r="F76" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G76" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H76" s="5" t="inlineStr">
+        <is>
+          <t>armor_penetration_percent → [10]</t>
+        </is>
+      </c>
+      <c r="I76" s="5" t="inlineStr">
+        <is>
+          <t>Vitesse, Vitesse</t>
+        </is>
+      </c>
+      <c r="J76" s="5" t="inlineStr">
+        <is>
+          <t>toutes</t>
+        </is>
+      </c>
+      <c r="K76" s="5" t="inlineStr">
+        <is>
+          <t>-80, -120</t>
+        </is>
+      </c>
+      <c r="L76" s="5" t="inlineStr">
+        <is>
+          <t>🗡️</t>
+        </is>
+      </c>
+      <c r="M76" s="5" t="inlineStr">
+        <is>
+          <t>Ignore 10% de la défense ennemie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>axe_or_1</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Bonus Or</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Utilité</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Passives</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="n">
+        <v>3</v>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>1,2,3</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>gold_drop_percent → [1,4,10]</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Confort</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>1224, 379</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>💰</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>axe_drop_1</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>Chance Drop</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>Utilité</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>Passives</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr"/>
+      <c r="F78" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G78" s="5" t="inlineStr">
+        <is>
+          <t>1,2,3</t>
+        </is>
+      </c>
+      <c r="H78" s="5" t="inlineStr">
+        <is>
+          <t>drop_rate_multiplier → [10,40,100]</t>
+        </is>
+      </c>
+      <c r="I78" s="5" t="inlineStr">
+        <is>
+          <t>Bonus Or, Bonus XP</t>
+        </is>
+      </c>
+      <c r="J78" s="5" t="inlineStr">
+        <is>
+          <t>toutes</t>
+        </is>
+      </c>
+      <c r="K78" s="5" t="inlineStr">
+        <is>
+          <t>1090, 530</t>
+        </is>
+      </c>
+      <c r="L78" s="5" t="inlineStr">
+        <is>
+          <t>🍀</t>
+        </is>
+      </c>
+      <c r="M78" s="5" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>axe_xp_1</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Bonus XP</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Utilité</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Passives</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="n">
+        <v>3</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>1,2,3</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>xp_drop_percent → [1,4,10]</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Confort</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>956, 379</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="inlineStr">
+        <is>
+          <t>axe_confort_1</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>Confort</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>Utilité</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>Passives</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr"/>
+      <c r="F80" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G80" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H80" s="5" t="inlineStr">
+        <is>
+          <t>unlock_feature → [tower_bonus_ticket]</t>
+        </is>
+      </c>
+      <c r="I80" s="5" t="inlineStr">
+        <is>
+          <t>Chance Drop</t>
+        </is>
+      </c>
+      <c r="J80" s="5" t="inlineStr"/>
+      <c r="K80" s="5" t="inlineStr">
+        <is>
+          <t>1090, 720</t>
+        </is>
+      </c>
+      <c r="L80" s="5" t="inlineStr">
+        <is>
+          <t>🎁</t>
+        </is>
+      </c>
+      <c r="M80" s="5" t="inlineStr">
+        <is>
+          <t>+1 ticket par jour pour la tour solo (non cumulable : 1 maximum par jour).</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>axe_or_2</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Bonus Or</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Utilité</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Passives</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="n">
+        <v>3</v>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>1,2,3</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>gold_drop_percent → [1,4,10]</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Confort</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>1224, 854</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>💰</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="inlineStr">
+        <is>
+          <t>axe_drop_2</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>Chance Drop</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>Utilité</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>Passives</t>
+        </is>
+      </c>
+      <c r="E82" s="5" t="inlineStr"/>
+      <c r="F82" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G82" s="5" t="inlineStr">
+        <is>
+          <t>1,2,3</t>
+        </is>
+      </c>
+      <c r="H82" s="5" t="inlineStr">
+        <is>
+          <t>drop_rate_multiplier → [10,40,100]</t>
+        </is>
+      </c>
+      <c r="I82" s="5" t="inlineStr">
+        <is>
+          <t>Bonus Or, Bonus XP</t>
+        </is>
+      </c>
+      <c r="J82" s="5" t="inlineStr">
+        <is>
+          <t>toutes</t>
+        </is>
+      </c>
+      <c r="K82" s="5" t="inlineStr">
+        <is>
+          <t>1090, 1005</t>
+        </is>
+      </c>
+      <c r="L82" s="5" t="inlineStr">
+        <is>
+          <t>🍀</t>
+        </is>
+      </c>
+      <c r="M82" s="5" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>axe_xp_2</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Bonus XP</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Utilité</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Passives</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="n">
+        <v>3</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>1,2,3</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>xp_drop_percent → [1,4,10]</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Confort</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>956, 854</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="5" t="inlineStr">
+        <is>
+          <t>axe_confort_2</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>Confort</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>Utilité</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>Passives</t>
+        </is>
+      </c>
+      <c r="E84" s="5" t="inlineStr"/>
+      <c r="F84" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G84" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H84" s="5" t="inlineStr">
+        <is>
+          <t>unlock_feature → [notify_events]</t>
+        </is>
+      </c>
+      <c r="I84" s="5" t="inlineStr">
+        <is>
+          <t>Chance Drop</t>
+        </is>
+      </c>
+      <c r="J84" s="5" t="inlineStr"/>
+      <c r="K84" s="5" t="inlineStr">
+        <is>
+          <t>1090, 1195</t>
+        </is>
+      </c>
+      <c r="L84" s="5" t="inlineStr">
+        <is>
+          <t>🎁</t>
+        </is>
+      </c>
+      <c r="M84" s="5" t="inlineStr">
+        <is>
+          <t>Reçois un message privé quand un événement apparaît.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M43"/>
+  <autoFilter ref="A1:M84"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(panoplies): bonus par rareté portée, comptage cumulatif, type choisi
Plus de familles d'objets : paliers 2 / 4 / 7 (×1 / ×1,5 / ×3) par rareté,
une pièce compte pour sa rareté et toutes celles en dessous (améliorer une
pièce ne fait jamais baisser le bonus), une deux-mains compte pour 2. Le
joueur choisit UN type de bonus avec /panoplie (players.panoplie_bonus).

Supprimés : sets.json, set_loader, /equiper_panoplie, EquipPanoplieUseCase,
PanoplieCraftsUseCase, pages admin des panoplies.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sakura_content.xlsx
+++ b/docs/sakura_content.xlsx
@@ -16,9 +16,8 @@
     <sheet name="🏪 Shop" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="🌳 Skill Tree" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="🏷️ Titres" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="🌸 Panoplies" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="🐉 World Bosses" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="⚙️ Calibrage" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="🐉 World Bosses" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="⚙️ Calibrage" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'🎽 Équipements'!$A$1:$T$24</definedName>
@@ -29,8 +28,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'🏪 Shop'!$A$1:$H$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'🌳 Skill Tree'!$A$1:$M$84</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'🏷️ Titres'!$A$1:$H$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'🌸 Panoplies'!$A$1:$I$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'🐉 World Bosses'!$A$1:$M$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'🐉 World Bosses'!$A$1:$M$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -496,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -513,7 +511,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 2026-10-23 23:07 UTC</t>
+          <t>Généré le 2026-10-24 12:41 UTC</t>
         </is>
       </c>
     </row>
@@ -616,93 +614,81 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>🌸 Panoplies</t>
+          <t>🐉 World Bosses</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Familles de set + paliers de bonus.</t>
+          <t>Bosses + modifiers.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>🐉 World Bosses</t>
+          <t>⚙️ Calibrage</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Bosses + modifiers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>⚙️ Calibrage</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
           <t>Constantes du score de puissance. NE PAS supprimer.</t>
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>🛠️ Comment équilibrer (round-trip)</t>
+        </is>
+      </c>
+    </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>🛠️ Comment équilibrer (round-trip)</t>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1. Filtre : clique la flèche d'un en-tête (ex : colonne Type = « Casque », ou Panoplie = « gobelin »).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1. Filtre : clique la flèche d'un en-tête (ex : colonne Type = « Casque », ou Panoplie = « gobelin »).</t>
+          <t>2. Édite les colonnes de stats (Atk, Def, PV, Crit %, Crit dmg, Esquive, Vitesse, Regen), le Prix, la Rareté, le Slot, la Panoplie, le Nom…</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2. Édite les colonnes de stats (Atk, Def, PV, Crit %, Crit dmg, Esquive, Vitesse, Regen), le Prix, la Rareté, le Slot, la Panoplie, le Nom…</t>
+          <t>3. La colonne « Power » (fond gris) est AUTO-CALCULÉE — ne l'édite pas, elle se met à jour toute seule quand tu changes une stat.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>3. La colonne « Power » (fond gris) est AUTO-CALCULÉE — ne l'édite pas, elle se met à jour toute seule quand tu changes une stat.</t>
+          <t>4. Tu peux AJOUTER une ligne d'équipement : remplis au moins Code + Type. Tu peux en supprimer aussi.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>4. Tu peux AJOUTER une ligne d'équipement : remplis au moins Code + Type. Tu peux en supprimer aussi.</t>
+          <t>5. Renvoie-moi le fichier .xlsx modifié → je réapplique via scripts/import_content_spreadsheet.py (puis seed + déploiement).</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>5. Renvoie-moi le fichier .xlsx modifié → je réapplique via scripts/import_content_spreadsheet.py (puis seed + déploiement).</t>
-        </is>
-      </c>
+      <c r="A21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Conventions stats : crit_chance &amp; esquive en 0..100 ; crit_damage 100 = neutre, 150 = ×1,5 ; défense soustractive (1 DEF ≈ 25 PV effectifs).</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
-        <is>
-          <t>Conventions stats : crit_chance &amp; esquive en 0..100 ; crit_damage 100 = neutre, 150 = ×1,5 ; défense soustractive (1 DEF ≈ 25 PV effectifs).</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
         <is>
           <t>Power d'un équipement = puissance MARGINALE qu'il ajoute à un perso de base (power(base+item) − power(base)).</t>
         </is>
@@ -714,79 +700,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Code famille</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>Nom</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>Icône</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>Items existants</t>
-        </is>
-      </c>
-      <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>Palier 2</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
-        <is>
-          <t>Palier 4</t>
-        </is>
-      </c>
-      <c r="H1" s="3" t="inlineStr">
-        <is>
-          <t>Palier 8</t>
-        </is>
-      </c>
-      <c r="I1" s="3" t="inlineStr">
-        <is>
-          <t>Palier 12</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:I1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1129,7 +1042,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3360,7 +3273,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Trouvaille — Tes chances de butin d'équipement sont augmentées de 10 % (1 % devient 1,1 %).</t>
+          <t>Trouvaille — Tes chances de butin d'équipement sont augmentées de 10 % (1 % devient 1,1 %), pour les raretés INFÉRIEURES à celle de cette pièce — jamais pour le mythique.</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
feat(pnj): Borak fusionne tout, Elna devient alchimiste (/alchimiste)
Borak fusionne aussi les accessoires (maîtrise d'Elna reportée sur lui).
Elna prépare les potions : ingrédients = matériaux de famille, confection
en or indexée sur le niveau, maîtrise en potions (remise, potion offerte).
Sept recettes : soins 10/35 %, mana 50 %, élixirs de récupération (régén
×3), force, garde, vitalité (+10 %, 1 h). Un même élixir se renouvelle,
des élixirs différents s'additionnent ; ils ne comptent qu'en combat de
zone et au world boss, interdits (et affichés) en épreuve et en défi.
Sorn ne vend plus de potions. /artisan remplacé par /alchimiste.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sakura_content.xlsx
+++ b/docs/sakura_content.xlsx
@@ -11,22 +11,24 @@
     <sheet name="🎽 Équipements" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="👹 Mobs" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="🧪 Consommables" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="📦 Ressources" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="🏪 Shop" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="🌳 Skill Tree" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="🏷️ Titres" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="🐉 World Bosses" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="⚙️ Calibrage" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="⚗️ Alchimie" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="📦 Ressources" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="🏪 Shop" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="🌳 Skill Tree" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="🏷️ Titres" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="🐉 World Bosses" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="⚙️ Calibrage" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'🎽 Équipements'!$A$1:$T$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'👹 Mobs'!$A$1:$S$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'🧪 Consommables'!$A$1:$H$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'📦 Ressources'!$A$1:$H$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'🏪 Shop'!$A$1:$H$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'🌳 Skill Tree'!$A$1:$M$87</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'🏷️ Titres'!$A$1:$H$29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'🐉 World Bosses'!$A$1:$M$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'🧪 Consommables'!$A$1:$H$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'⚗️ Alchimie'!$A$1:$F$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'📦 Ressources'!$A$1:$H$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'🏪 Shop'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'🌳 Skill Tree'!$A$1:$M$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'🏷️ Titres'!$A$1:$H$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'🐉 World Bosses'!$A$1:$M$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -492,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -509,7 +511,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 2026-10-25 16:07 UTC</t>
+          <t>Généré le 2026-10-26 07:25 UTC</t>
         </is>
       </c>
     </row>
@@ -557,124 +559,136 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Potions et ressources de craft.</t>
+          <t>Potions et matériaux de famille.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>🏪 Shop</t>
+          <t>⚗️ Alchimie</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Prix d'achat / vente du shop.</t>
+          <t>Recettes d'Elna : ingrédients, or de confection, maîtrise.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>🌳 Skill Tree</t>
+          <t>🏪 Shop</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Tous les nœuds de l'arbre.</t>
+          <t>Prix d'achat / vente du shop.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>🏷️ Titres</t>
+          <t>🌳 Skill Tree</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Titres, conditions et effets.</t>
+          <t>Tous les nœuds de l'arbre.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>🐉 World Bosses</t>
+          <t>🏷️ Titres</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Bosses + modifiers.</t>
+          <t>Titres, conditions et effets.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>🐉 World Bosses</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Bosses + modifiers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>⚙️ Calibrage</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Constantes du score de puissance. NE PAS supprimer.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>🛠️ Comment équilibrer (round-trip)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>1. Filtre : clique la flèche d'un en-tête (ex : colonne Type = « Casque », ou Panoplie = « gobelin »).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2. Édite les colonnes de stats (Atk, Def, PV, Crit %, Crit dmg, Esquive, Vitesse, Regen), le Prix, la Rareté, le Slot, la Panoplie, le Nom…</t>
+          <t>1. Filtre : clique la flèche d'un en-tête (ex : colonne Type = « Casque », ou Panoplie = « gobelin »).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>3. La colonne « Power » (fond gris) est AUTO-CALCULÉE — ne l'édite pas, elle se met à jour toute seule quand tu changes une stat.</t>
+          <t>2. Édite les colonnes de stats (Atk, Def, PV, Crit %, Crit dmg, Esquive, Vitesse, Regen), le Prix, la Rareté, le Slot, la Panoplie, le Nom…</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>4. Tu peux AJOUTER une ligne d'équipement : remplis au moins Code + Type. Tu peux en supprimer aussi.</t>
+          <t>3. La colonne « Power » (fond gris) est AUTO-CALCULÉE — ne l'édite pas, elle se met à jour toute seule quand tu changes une stat.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>4. Tu peux AJOUTER une ligne d'équipement : remplis au moins Code + Type. Tu peux en supprimer aussi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>5. Renvoie-moi le fichier .xlsx modifié → je réapplique via scripts/import_content_spreadsheet.py (puis seed + déploiement).</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr"/>
-    </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Conventions stats : crit_chance &amp; esquive en 0..100 ; crit_damage 100 = neutre, 150 = ×1,5 ; défense soustractive (1 DEF ≈ 25 PV effectifs).</t>
-        </is>
-      </c>
+      <c r="A21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
+        <is>
+          <t>Conventions stats : crit_chance &amp; esquive en 0..100 ; crit_damage 100 = neutre, 150 = ×1,5 ; défense soustractive (1 DEF ≈ 25 PV effectifs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>Power d'un équipement = puissance MARGINALE qu'il ajoute à un perso de base (power(base+item) − power(base)).</t>
         </is>
@@ -686,6 +700,349 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="48" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="48" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Nom</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Famille</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>PV max</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Def</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Vit</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Crit %</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Crit dmg</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>Esquive</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>Modifiers</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>Poids spawn</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>Lore</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>slime_titan</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Titan Visqueux</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr"/>
+      <c r="D2" s="5" t="n">
+        <v>13000</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>110</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="J2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="7" t="inlineStr">
+        <is>
+          <t>damage_immunity_threshold = 5
+auto_heal_per_turn = 32</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>Un slime ancestral devenu colosse, sa masse étouffante absorbe les coups les plus faibles et se régénère lentement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>gobelin_warlord</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Seigneur de Guerre Gobelin</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="n">
+        <v>16000</v>
+      </c>
+      <c r="E3" t="n">
+        <v>212</v>
+      </c>
+      <c r="F3" t="n">
+        <v>16</v>
+      </c>
+      <c r="G3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I3" t="n">
+        <v>130</v>
+      </c>
+      <c r="J3" t="n">
+        <v>5</v>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>enrage_below_pct = 30
+enrage_attack_multiplier = 1.5
+adds = {'attack': 148, 'summon_turn_interval': 4, 'max_active': 3}</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>8</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Le chef d'une horde sanguinaire. Plus il est blessé, plus sa rage l'amplifie, et il appelle des renforts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>stone_colossus</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Colosse de Pierre</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="n">
+        <v>209000</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>damage_immunity_threshold = 27
+reflect_pct = 15</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>Une statue runique animée par d'antiques magies. Inébranlable face aux frappes faibles, sa carapace renvoie une part des coups.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>shadow_wraith</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Spectre des Ténèbres</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="n">
+        <v>186000</v>
+      </c>
+      <c r="E5" t="n">
+        <v>473</v>
+      </c>
+      <c r="F5" t="n">
+        <v>30</v>
+      </c>
+      <c r="G5" t="n">
+        <v>18</v>
+      </c>
+      <c r="H5" t="n">
+        <v>10</v>
+      </c>
+      <c r="I5" t="n">
+        <v>150</v>
+      </c>
+      <c r="J5" t="n">
+        <v>30</v>
+      </c>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>crit_immunity = True
+phases = [{'below_pct': 50, 'attack_multiplier': 1.3}, {'below_pct': 20, 'attack_multiplier': 1.6}]</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>2</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Une entité incorporelle qui glisse entre les coups. Les coups critiques traversent sa forme étherée, et il mute en s'affaiblissant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>ancient_dragon</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Dragon Ancestral</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="n">
+        <v>111000</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>585</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>200</v>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>damage_immunity_threshold = 43
+enrage_below_pct = 25
+enrage_attack_multiplier = 1.8
+auto_heal_per_turn = 179
+reflect_pct = 20
+adds = {'attack': 351, 'summon_turn_interval': 5, 'max_active': 2}
+phases = [{'below_pct': 50, 'attack_multiplier': 1.25}]</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>Le sommet de l'évolution. Inflige des coups dévastateurs, renvoie les frappes, invoque des drakelings, se régénère et entre en rage à la fin.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:M6"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8531,11 +8888,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -8611,24 +8968,600 @@
         <v>10</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>Rend 10% des PV max (sans dépasser le maximum).</t>
+          <t>Rend 10 % des PV max (sans dépasser le maximum). Préparée par Elna, l'alchimiste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>potion_soin_superieure</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Potion de soin supérieure</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>heal_percent</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>35</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Rend 35 % des PV max (sans dépasser le maximum).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>potion_mana</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Potion de mana</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>mana_percent</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Rend 50 % du mana max (sans dépasser le maximum).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>elixir_recuperation</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Élixir de récupération</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>elixir</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Pendant 1 h, tes PV et ton mana remontent 3 fois plus vite hors combat. Le reboire renouvelle sa durée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>elixir_force</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Élixir de force</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>elixir</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>+10 % d'attaque pendant 1 h, en combat de zone et au world boss (pas en épreuve ni en défi). Le reboire renouvelle sa durée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>elixir_garde</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Élixir de garde</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>elixir</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>+10 % de défense pendant 1 h, en combat de zone et au world boss (pas en épreuve ni en défi). Le reboire renouvelle sa durée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>elixir_vitalite</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Élixir de vitalité</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>elixir</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>+10 % de PV max pendant 1 h, en combat de zone et au world boss (pas en épreuve ni en défi). Le reboire renouvelle sa durée.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H2"/>
+  <autoFilter ref="A1:H8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Potion</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Effet</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Ingrédients</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Or × niveau</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Or au niveau 50</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Potion de soin</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>potion_soin</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>rend 10 % de tes PV</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>2 × Gelée</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Potion de soin supérieure</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>potion_soin_superieure</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>rend 35 % de tes PV</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>4 × Gelée + 2 × Dent de gobelin</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Potion de mana</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>potion_mana</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>rend 50 % de ton mana</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>3 × Fragment d'âme</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Élixir de récupération</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>elixir_recuperation</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>régénération des PV et du mana ×3 hors combat pendant 1 h</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>3 × Dent de gobelin + 2 × Fragment d'âme</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F5" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Élixir de force</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>elixir_force</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+10 % d'attaque pendant 1 h (combats de zone et world boss)</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>3 × Cœur corrompu</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Élixir de garde</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>elixir_garde</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>+10 % de défense pendant 1 h (combats de zone et world boss)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2 × Cœur corrompu + 2 × Fragment d'âme</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F7" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Élixir de vitalité</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>elixir_vitalite</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+10 % de PV max pendant 1 h (combats de zone et world boss)</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>2 × Cœur corrompu + 2 × Dent de gobelin</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Maîtrise</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Potions préparées</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Remise</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Potion offerte</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Apprentie</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>0 %</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>0 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Compagne</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>5 %</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>0 %</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="5" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Maîtresse</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>120</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Légendaire</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>400</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>15 %</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>20 %</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="n"/>
+      <c r="F14" s="5" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F14"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8983,17 +9916,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -9044,47 +9977,13 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>potion_soin</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>Potion de soin</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>consumable</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="n">
-        <v>20</v>
-      </c>
-      <c r="E2" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="F2" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="G2" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H2"/>
+  <autoFilter ref="A1:H1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13933,7 +14832,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15179,347 +16078,4 @@
   <autoFilter ref="A1:H29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="48" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="48" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>Nom</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>Famille</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>PV max</t>
-        </is>
-      </c>
-      <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>Atk</t>
-        </is>
-      </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>Def</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
-        <is>
-          <t>Vit</t>
-        </is>
-      </c>
-      <c r="H1" s="3" t="inlineStr">
-        <is>
-          <t>Crit %</t>
-        </is>
-      </c>
-      <c r="I1" s="3" t="inlineStr">
-        <is>
-          <t>Crit dmg</t>
-        </is>
-      </c>
-      <c r="J1" s="3" t="inlineStr">
-        <is>
-          <t>Esquive</t>
-        </is>
-      </c>
-      <c r="K1" s="3" t="inlineStr">
-        <is>
-          <t>Modifiers</t>
-        </is>
-      </c>
-      <c r="L1" s="3" t="inlineStr">
-        <is>
-          <t>Poids spawn</t>
-        </is>
-      </c>
-      <c r="M1" s="3" t="inlineStr">
-        <is>
-          <t>Lore</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>slime_titan</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>Titan Visqueux</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr"/>
-      <c r="D2" s="5" t="n">
-        <v>13000</v>
-      </c>
-      <c r="E2" s="5" t="n">
-        <v>110</v>
-      </c>
-      <c r="F2" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="G2" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="H2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="J2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" s="7" t="inlineStr">
-        <is>
-          <t>damage_immunity_threshold = 5
-auto_heal_per_turn = 32</t>
-        </is>
-      </c>
-      <c r="L2" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="M2" s="5" t="inlineStr">
-        <is>
-          <t>Un slime ancestral devenu colosse, sa masse étouffante absorbe les coups les plus faibles et se régénère lentement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>gobelin_warlord</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Seigneur de Guerre Gobelin</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="n">
-        <v>16000</v>
-      </c>
-      <c r="E3" t="n">
-        <v>212</v>
-      </c>
-      <c r="F3" t="n">
-        <v>16</v>
-      </c>
-      <c r="G3" t="n">
-        <v>12</v>
-      </c>
-      <c r="H3" t="n">
-        <v>5</v>
-      </c>
-      <c r="I3" t="n">
-        <v>130</v>
-      </c>
-      <c r="J3" t="n">
-        <v>5</v>
-      </c>
-      <c r="K3" s="8" t="inlineStr">
-        <is>
-          <t>enrage_below_pct = 30
-enrage_attack_multiplier = 1.5
-adds = {'attack': 148, 'summon_turn_interval': 4, 'max_active': 3}</t>
-        </is>
-      </c>
-      <c r="L3" t="n">
-        <v>8</v>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Le chef d'une horde sanguinaire. Plus il est blessé, plus sa rage l'amplifie, et il appelle des renforts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>stone_colossus</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Colosse de Pierre</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="n">
-        <v>209000</v>
-      </c>
-      <c r="E4" s="5" t="n">
-        <v>350</v>
-      </c>
-      <c r="F4" s="5" t="n">
-        <v>23</v>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="H4" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="J4" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="7" t="inlineStr">
-        <is>
-          <t>damage_immunity_threshold = 27
-reflect_pct = 15</t>
-        </is>
-      </c>
-      <c r="L4" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="M4" s="5" t="inlineStr">
-        <is>
-          <t>Une statue runique animée par d'antiques magies. Inébranlable face aux frappes faibles, sa carapace renvoie une part des coups.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>shadow_wraith</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Spectre des Ténèbres</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="n">
-        <v>186000</v>
-      </c>
-      <c r="E5" t="n">
-        <v>473</v>
-      </c>
-      <c r="F5" t="n">
-        <v>30</v>
-      </c>
-      <c r="G5" t="n">
-        <v>18</v>
-      </c>
-      <c r="H5" t="n">
-        <v>10</v>
-      </c>
-      <c r="I5" t="n">
-        <v>150</v>
-      </c>
-      <c r="J5" t="n">
-        <v>30</v>
-      </c>
-      <c r="K5" s="8" t="inlineStr">
-        <is>
-          <t>crit_immunity = True
-phases = [{'below_pct': 50, 'attack_multiplier': 1.3}, {'below_pct': 20, 'attack_multiplier': 1.6}]</t>
-        </is>
-      </c>
-      <c r="L5" t="n">
-        <v>2</v>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Une entité incorporelle qui glisse entre les coups. Les coups critiques traversent sa forme étherée, et il mute en s'affaiblissant.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>ancient_dragon</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Dragon Ancestral</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="n">
-        <v>111000</v>
-      </c>
-      <c r="E6" s="5" t="n">
-        <v>585</v>
-      </c>
-      <c r="F6" s="5" t="n">
-        <v>37</v>
-      </c>
-      <c r="G6" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="H6" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="I6" s="5" t="n">
-        <v>200</v>
-      </c>
-      <c r="J6" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="K6" s="7" t="inlineStr">
-        <is>
-          <t>damage_immunity_threshold = 43
-enrage_below_pct = 25
-enrage_attack_multiplier = 1.8
-auto_heal_per_turn = 179
-reflect_pct = 20
-adds = {'attack': 351, 'summon_turn_interval': 5, 'max_active': 2}
-phases = [{'below_pct': 50, 'attack_multiplier': 1.25}]</t>
-        </is>
-      </c>
-      <c r="L6" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="M6" s="5" t="inlineStr">
-        <is>
-          <t>Le sommet de l'évolution. Inflige des coups dévastateurs, renvoie les frappes, invoque des drakelings, se régénère et entre en rage à la fin.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:M6"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(sorn): étal d'outils et cosmétiques de profil (/apparence)
Sorn vend des outils et des cosmétiques, à prix fixes identiques pour
tous (par rang/zone quand l'effet grandit) : cor de chasse par zone
(invoque l'élite après le combat en cours, 1 h entre deux cors), sceau
du second souffle par rang (efface l'attente d'épreuve), parchemin
d'oubli et jeton d'arbre (150 / 60 × niveau, un seul à la fois),
sablier de fidélité (pardonne un jour de /daily manqué). 16 cosmétiques
(fonds, cadres, couleurs de titre) portés sur /profil via /apparence.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sakura_content.xlsx
+++ b/docs/sakura_content.xlsx
@@ -22,10 +22,10 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'🎽 Équipements'!$A$1:$T$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'👹 Mobs'!$A$1:$S$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'🧪 Consommables'!$A$1:$H$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'🧪 Consommables'!$A$1:$H$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'⚗️ Alchimie'!$A$1:$F$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'📦 Ressources'!$A$1:$H$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'🏪 Shop'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'🏪 Shop'!$A$1:$I$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'🌳 Skill Tree'!$A$1:$M$87</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'🏷️ Titres'!$A$1:$H$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'🐉 World Bosses'!$A$1:$M$6</definedName>
@@ -511,7 +511,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 2026-10-26 07:25 UTC</t>
+          <t>Généré le 2026-10-26 10:11 UTC</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Prix d'achat / vente du shop.</t>
+          <t>L'étal de Sorn : outils (cor, sceau, parchemin, jeton, sablier) et cosmétiques.</t>
         </is>
       </c>
     </row>
@@ -8888,11 +8888,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -9195,8 +9195,484 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>cor_chasse_f</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Cor de chasse de la Clairière</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>summon_elite</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Fait apparaître l'élite de la Clairière sinistre (rang F) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>cor_chasse_e</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Cor de chasse du Cimetière</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>summon_elite</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr"/>
+      <c r="F10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Fait apparaître l'élite de le Cimetière abandonné (rang E) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>cor_chasse_d</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Cor de chasse du Berceau</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>summon_elite</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Fait apparaître l'élite de le Berceau cataclysmique (rang D) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>sceau_souffle_e</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Sceau du second souffle (rang E)</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>trial_retry</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr"/>
+      <c r="F12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Efface l'attente après un échec à l'épreuve du rang E : tu peux la retenter tout de suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>sceau_souffle_d</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Sceau du second souffle (rang D)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>trial_retry</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Efface l'attente après un échec à l'épreuve du rang D : tu peux la retenter tout de suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>sceau_souffle_c</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Sceau du second souffle (rang C)</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>trial_retry</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr"/>
+      <c r="F14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Efface l'attente après un échec à l'épreuve du rang C : tu peux la retenter tout de suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>sceau_souffle_b</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Sceau du second souffle (rang B)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>trial_retry</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Efface l'attente après un échec à l'épreuve du rang B : tu peux la retenter tout de suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>sceau_souffle_a</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Sceau du second souffle (rang A)</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>trial_retry</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr"/>
+      <c r="F16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Efface l'attente après un échec à l'épreuve du rang A : tu peux la retenter tout de suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>sceau_souffle_s</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Sceau du second souffle (rang S)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>trial_retry</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Efface l'attente après un échec à l'épreuve du rang S : tu peux la retenter tout de suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>sceau_souffle_ss</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Sceau du second souffle (rang SS)</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>trial_retry</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr"/>
+      <c r="F18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Efface l'attente après un échec à l'épreuve du rang SS : tu peux la retenter tout de suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>sceau_souffle_sss</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Sceau du second souffle (rang SSS)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>trial_retry</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Efface l'attente après un échec à l'épreuve du rang SSS : tu peux la retenter tout de suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>parchemin_oubli</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Parchemin d'oubli</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>respec_stats</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr"/>
+      <c r="F20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Reprend TOUS tes points de stats (attaque, défense, PV) : replace-les ensuite avec /stats.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>jeton_arbre</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Jeton de réinitialisation d'arbre</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>reset_tree</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Réinitialise ton arbre de compétences EN PLUS du reset gratuit de la semaine (à garder pour quand il est déjà pris).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>sablier_fidelite</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Sablier de fidélité</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>daily_guard</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr"/>
+      <c r="F22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>Le premier jour de /daily manqué, ta série n'est pas divisée par deux. Il agit tout seul ; un seul à la fois.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H8"/>
+  <autoFilter ref="A1:H22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9922,17 +10398,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -9953,22 +10430,22 @@
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
+          <t>Rareté</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
           <t>Prix achat</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>Prix vente max</t>
-        </is>
-      </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>Prix vente min</t>
+          <t>Prix × niveau</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>Seuil stock</t>
+          <t>Un seul à la fois</t>
         </is>
       </c>
       <c r="H1" s="3" t="inlineStr">
@@ -9976,9 +10453,1364 @@
           <t>Activé</t>
         </is>
       </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>cor_chasse_f</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Cor de chasse de la Clairière</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>Fait apparaître l'élite de la Clairière sinistre (rang F) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>cor_chasse_e</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Cor de chasse du Cimetière</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Fait apparaître l'élite de le Cimetière abandonné (rang E) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>cor_chasse_d</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Cor de chasse du Berceau</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>2600</v>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Fait apparaître l'élite de le Berceau cataclysmique (rang D) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>sceau_souffle_e</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Sceau du second souffle (rang E)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>700</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Efface l'attente après un échec à l'épreuve du rang E : tu peux la retenter tout de suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>sceau_souffle_d</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Sceau du second souffle (rang D)</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Efface l'attente après un échec à l'épreuve du rang D : tu peux la retenter tout de suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>sceau_souffle_c</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Sceau du second souffle (rang C)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>2300</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Efface l'attente après un échec à l'épreuve du rang C : tu peux la retenter tout de suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>sceau_souffle_b</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Sceau du second souffle (rang B)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Efface l'attente après un échec à l'épreuve du rang B : tu peux la retenter tout de suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>sceau_souffle_a</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Sceau du second souffle (rang A)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>3800</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Efface l'attente après un échec à l'épreuve du rang A : tu peux la retenter tout de suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>sceau_souffle_s</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Sceau du second souffle (rang S)</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>4500</v>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Efface l'attente après un échec à l'épreuve du rang S : tu peux la retenter tout de suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>sceau_souffle_ss</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Sceau du second souffle (rang SS)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>5300</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Efface l'attente après un échec à l'épreuve du rang SS : tu peux la retenter tout de suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>sceau_souffle_sss</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Sceau du second souffle (rang SSS)</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>6000</v>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>Efface l'attente après un échec à l'épreuve du rang SSS : tu peux la retenter tout de suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>parchemin_oubli</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Parchemin d'oubli</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>150</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Reprend TOUS tes points de stats (attaque, défense, PV) : replace-les ensuite avec /stats.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>jeton_arbre</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Jeton de réinitialisation d'arbre</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Réinitialise ton arbre de compétences EN PLUS du reset gratuit de la semaine (à garder pour quand il est déjà pris).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>sablier_fidelite</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Sablier de fidélité</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Le premier jour de /daily manqué, ta série n'est pas divisée par deux. Il agit tout seul ; un seul à la fois.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>fond_aube_rosee</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Fond — Aube rosée</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>cosmetic</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Cosmétique : change le fond de ta bannière /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>fond_foret_emeraude</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Fond — Forêt d'émeraude</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>cosmetic</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Cosmétique : change le fond de ta bannière /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>fond_ocean_profond</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Fond — Océan profond</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>cosmetic</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>Cosmétique : change le fond de ta bannière /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>fond_braises</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Fond — Braises du Berceau</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>cosmetic</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Cosmétique : change le fond de ta bannière /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>fond_crepuscule_dore</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Fond — Crépuscule doré</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>cosmetic</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>epic</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>40000</v>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Cosmétique : change le fond de ta bannière /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>fond_aurore_boreale</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Fond — Aurore boréale</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>cosmetic</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>legendary</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>150000</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Cosmétique : change le fond de ta bannière /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>cadre_argent</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Cadre — Argent</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>cosmetic</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>Cosmétique : change l'anneau autour de ton avatar sur /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>cadre_jade</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Cadre — Jade</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>cosmetic</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Cosmétique : change l'anneau autour de ton avatar sur /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>cadre_amethyste</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Cadre — Améthyste</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>cosmetic</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>Cosmétique : change l'anneau autour de ton avatar sur /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>cadre_or_royal</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Cadre — Or royal</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>cosmetic</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>epic</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>40000</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Cosmétique : change l'anneau autour de ton avatar sur /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>cadre_sakura_eternel</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Cadre — Sakura éternel</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>cosmetic</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>legendary</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v>150000</v>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>Cosmétique : change l'anneau autour de ton avatar sur /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>titre_ivoire</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Titre — Ivoire</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>cosmetic</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Cosmétique : change la couleur de ton titre sur /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>titre_azur</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Titre — Azur</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>cosmetic</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>Cosmétique : change la couleur de ton titre sur /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>titre_emeraude</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Titre — Émeraude</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>cosmetic</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Cosmétique : change la couleur de ton titre sur /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>titre_rubis</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Titre — Rubis</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>cosmetic</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>epic</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>40000</v>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>Cosmétique : change la couleur de ton titre sur /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>titre_or_flamboyant</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Titre — Or flamboyant</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>cosmetic</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>legendary</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>150000</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Cosmétique : change la couleur de ton titre sur /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:I31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(contenu): titres de chasse pour toutes les zones, potions supérieures, ouverture des zones en une commande
- 47 titres : un Pourfendeur par famille, un Chasseur légendaire par
  monstre (25 victoires pour une élite) ;
- Elna : 6 potions supérieures avec les matériaux des zones C, B, A ; un
  élixir plus fort remplace le plus faible, jamais l'inverse ;
- cors de chasse C/B/A (inactifs jusqu'à l'ouverture de leur zone) ;
- scripts/open_zones : ouvre les zones, recale les familles, recalibre
  les élites, active les cors et recalcule leurs prix ;
- articles de Sorn gérés par le contenu (prix synchronisés au seed).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sakura_content.xlsx
+++ b/docs/sakura_content.xlsx
@@ -22,12 +22,12 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'🎽 Équipements'!$A$1:$T$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'👹 Mobs'!$A$1:$S$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'🧪 Consommables'!$A$1:$H$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'⚗️ Alchimie'!$A$1:$F$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'🧪 Consommables'!$A$1:$H$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'⚗️ Alchimie'!$A$1:$F$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'📦 Ressources'!$A$1:$H$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'🏪 Shop'!$A$1:$I$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'🏪 Shop'!$A$1:$I$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'🌳 Skill Tree'!$A$1:$M$87</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'🏷️ Titres'!$A$1:$H$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'🏷️ Titres'!$A$1:$H$76</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'🐉 World Bosses'!$A$1:$M$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -511,7 +511,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 2026-10-26 10:11 UTC</t>
+          <t>Généré le 2026-10-26 13:23 UTC</t>
         </is>
       </c>
     </row>
@@ -8888,10 +8888,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
@@ -9198,12 +9198,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>cor_chasse_f</t>
+          <t>grande_potion_soin</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Cor de chasse de la Clairière</t>
+          <t>Grande potion de soin</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -9213,10 +9213,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>summon_elite</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
+          <t>heal_percent</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>60</v>
+      </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
@@ -9225,19 +9227,19 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Fait apparaître l'élite de la Clairière sinistre (rang F) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
+          <t>Rend 60 % des PV max (sans dépasser le maximum).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>cor_chasse_e</t>
+          <t>grande_potion_mana</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Cor de chasse du Cimetière</t>
+          <t>Grande potion de mana</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -9247,10 +9249,12 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>summon_elite</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr"/>
+          <t>mana_percent</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>100</v>
+      </c>
       <c r="F10" s="5" t="n">
         <v>0</v>
       </c>
@@ -9259,19 +9263,19 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Fait apparaître l'élite de le Cimetière abandonné (rang E) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
+          <t>Rend tout le mana.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>cor_chasse_d</t>
+          <t>elixir_recuperation_sup</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Cor de chasse du Berceau</t>
+          <t>Élixir de récupération supérieur</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -9281,10 +9285,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>summon_elite</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
+          <t>elixir</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>5</v>
+      </c>
       <c r="F11" t="n">
         <v>0</v>
       </c>
@@ -9293,19 +9299,19 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Fait apparaître l'élite de le Berceau cataclysmique (rang D) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
+          <t>Pendant 1 h, tes PV et ton mana remontent 5 fois plus vite hors combat. Le reboire renouvelle sa durée ; un élixir plus faible du même type ne le remplace pas.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>sceau_souffle_e</t>
+          <t>elixir_force_sup</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Sceau du second souffle (rang E)</t>
+          <t>Élixir de force supérieur</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -9315,10 +9321,12 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>trial_retry</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr"/>
+          <t>elixir</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>20</v>
+      </c>
       <c r="F12" s="5" t="n">
         <v>0</v>
       </c>
@@ -9327,19 +9335,19 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Efface l'attente après un échec à l'épreuve du rang E : tu peux la retenter tout de suite.</t>
+          <t>+20 % d'attaque pendant 1 h, en combat de zone et au world boss (pas en épreuve ni en défi). Le reboire renouvelle sa durée ; un élixir plus faible du même type ne le remplace pas.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>sceau_souffle_d</t>
+          <t>elixir_garde_sup</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Sceau du second souffle (rang D)</t>
+          <t>Élixir de garde supérieur</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -9349,10 +9357,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>trial_retry</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
+          <t>elixir</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>20</v>
+      </c>
       <c r="F13" t="n">
         <v>0</v>
       </c>
@@ -9361,19 +9371,19 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Efface l'attente après un échec à l'épreuve du rang D : tu peux la retenter tout de suite.</t>
+          <t>+20 % de défense pendant 1 h, en combat de zone et au world boss (pas en épreuve ni en défi). Le reboire renouvelle sa durée ; un élixir plus faible du même type ne le remplace pas.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>sceau_souffle_c</t>
+          <t>elixir_vitalite_sup</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Sceau du second souffle (rang C)</t>
+          <t>Élixir de vitalité supérieur</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -9383,10 +9393,12 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>trial_retry</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr"/>
+          <t>elixir</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>20</v>
+      </c>
       <c r="F14" s="5" t="n">
         <v>0</v>
       </c>
@@ -9395,19 +9407,19 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>Efface l'attente après un échec à l'épreuve du rang C : tu peux la retenter tout de suite.</t>
+          <t>+20 % de PV max pendant 1 h, en combat de zone et au world boss (pas en épreuve ni en défi). Le reboire renouvelle sa durée ; un élixir plus faible du même type ne le remplace pas.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>sceau_souffle_b</t>
+          <t>cor_chasse_f</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Sceau du second souffle (rang B)</t>
+          <t>Cor de chasse de la Clairière</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -9417,7 +9429,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>trial_retry</t>
+          <t>summon_elite</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
@@ -9429,19 +9441,19 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Efface l'attente après un échec à l'épreuve du rang B : tu peux la retenter tout de suite.</t>
+          <t>Fait apparaître l'élite de la Clairière sinistre (rang F) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>sceau_souffle_a</t>
+          <t>cor_chasse_e</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Sceau du second souffle (rang A)</t>
+          <t>Cor de chasse du Cimetière</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -9451,7 +9463,7 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>trial_retry</t>
+          <t>summon_elite</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr"/>
@@ -9463,19 +9475,19 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Efface l'attente après un échec à l'épreuve du rang A : tu peux la retenter tout de suite.</t>
+          <t>Fait apparaître l'élite du Cimetière abandonné (rang E) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>sceau_souffle_s</t>
+          <t>cor_chasse_d</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Sceau du second souffle (rang S)</t>
+          <t>Cor de chasse du Berceau</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -9485,7 +9497,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>trial_retry</t>
+          <t>summon_elite</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
@@ -9497,19 +9509,19 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Efface l'attente après un échec à l'épreuve du rang S : tu peux la retenter tout de suite.</t>
+          <t>Fait apparaître l'élite du Berceau cataclysmique (rang D) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>sceau_souffle_ss</t>
+          <t>cor_chasse_c</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Sceau du second souffle (rang SS)</t>
+          <t>Cor de chasse du Sanctuaire</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -9519,7 +9531,7 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>trial_retry</t>
+          <t>summon_elite</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr"/>
@@ -9531,19 +9543,19 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Efface l'attente après un échec à l'épreuve du rang SS : tu peux la retenter tout de suite.</t>
+          <t>Fait apparaître l'élite du Sanctuaire primordial (rang C) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>sceau_souffle_sss</t>
+          <t>cor_chasse_b</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Sceau du second souffle (rang SSS)</t>
+          <t>Cor de chasse de l'Éclipse</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -9553,7 +9565,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>trial_retry</t>
+          <t>summon_elite</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
@@ -9565,19 +9577,19 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Efface l'attente après un échec à l'épreuve du rang SSS : tu peux la retenter tout de suite.</t>
+          <t>Fait apparaître l'élite de l'Éclipse éternelle (rang B) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>parchemin_oubli</t>
+          <t>cor_chasse_a</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Parchemin d'oubli</t>
+          <t>Cor de chasse des Cimes</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -9587,7 +9599,7 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>respec_stats</t>
+          <t>summon_elite</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr"/>
@@ -9599,19 +9611,19 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Reprend TOUS tes points de stats (attaque, défense, PV) : replace-les ensuite avec /stats.</t>
+          <t>Fait apparaître l'élite des Cimes des Wyrms (rang A) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>jeton_arbre</t>
+          <t>sceau_souffle_e</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Jeton de réinitialisation d'arbre</t>
+          <t>Sceau du second souffle (rang E)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -9621,7 +9633,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>reset_tree</t>
+          <t>trial_retry</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
@@ -9633,19 +9645,19 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Réinitialise ton arbre de compétences EN PLUS du reset gratuit de la semaine (à garder pour quand il est déjà pris).</t>
+          <t>Efface l'attente après un échec à l'épreuve du rang E : tu peux la retenter tout de suite.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>sablier_fidelite</t>
+          <t>sceau_souffle_d</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Sablier de fidélité</t>
+          <t>Sceau du second souffle (rang D)</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -9655,7 +9667,7 @@
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>daily_guard</t>
+          <t>trial_retry</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr"/>
@@ -9667,12 +9679,318 @@
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
+          <t>Efface l'attente après un échec à l'épreuve du rang D : tu peux la retenter tout de suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>sceau_souffle_c</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Sceau du second souffle (rang C)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>trial_retry</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Efface l'attente après un échec à l'épreuve du rang C : tu peux la retenter tout de suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>sceau_souffle_b</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Sceau du second souffle (rang B)</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>trial_retry</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr"/>
+      <c r="F24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>Efface l'attente après un échec à l'épreuve du rang B : tu peux la retenter tout de suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>sceau_souffle_a</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Sceau du second souffle (rang A)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>trial_retry</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Efface l'attente après un échec à l'épreuve du rang A : tu peux la retenter tout de suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>sceau_souffle_s</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Sceau du second souffle (rang S)</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>trial_retry</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr"/>
+      <c r="F26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>Efface l'attente après un échec à l'épreuve du rang S : tu peux la retenter tout de suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>sceau_souffle_ss</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Sceau du second souffle (rang SS)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>trial_retry</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Efface l'attente après un échec à l'épreuve du rang SS : tu peux la retenter tout de suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>sceau_souffle_sss</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Sceau du second souffle (rang SSS)</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>trial_retry</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr"/>
+      <c r="F28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>Efface l'attente après un échec à l'épreuve du rang SSS : tu peux la retenter tout de suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>parchemin_oubli</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Parchemin d'oubli</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>respec_stats</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Reprend TOUS tes points de stats (attaque, défense, PV) : replace-les ensuite avec /stats.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>jeton_arbre</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Jeton de réinitialisation d'arbre</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>reset_tree</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr"/>
+      <c r="F30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>Réinitialise ton arbre de compétences EN PLUS du reset gratuit de la semaine (à garder pour quand il est déjà pris).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>sablier_fidelite</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Sablier de fidélité</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>daily_guard</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
           <t>Le premier jour de /daily manqué, ta série n'est pas divisée par deux. Il agit tout seul ; un seul à la fois.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H22"/>
+  <autoFilter ref="A1:H31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9683,13 +10001,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
   </cols>
@@ -9922,117 +10240,285 @@
         <v>500</v>
       </c>
     </row>
-    <row r="9"/>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Grande potion de soin</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>grande_potion_soin</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>rend 60 % de tes PV</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>3 × Croc primordial</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F9" t="n">
+        <v>300</v>
+      </c>
+    </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Maîtrise</t>
+          <t>Grande potion de mana</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Potions préparées</t>
+          <t>grande_potion_mana</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Remise</t>
+          <t>rend 100 % de ton mana</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Potion offerte</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
+          <t>3 × Sang lunaire</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>250</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Apprentie</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>0</v>
+          <t>Élixir de récupération supérieur</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>elixir_recuperation_sup</t>
+        </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0 %</t>
+          <t>régénération des PV et du mana ×5 hors combat pendant 1 h</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0 %</t>
-        </is>
+          <t>3 × Sang lunaire + 2 × Croc primordial</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>9</v>
+      </c>
+      <c r="F11" t="n">
+        <v>450</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Compagne</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="n">
-        <v>30</v>
+          <t>Élixir de force supérieur</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>elixir_force_sup</t>
+        </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>5 %</t>
+          <t>+20 % d'attaque pendant 1 h (combats de zone et world boss)</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>0 %</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
+          <t>3 × Écaille de dragon</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>750</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Maîtresse</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>120</v>
+          <t>Élixir de garde supérieur</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>elixir_garde_sup</t>
+        </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>10 %</t>
+          <t>+20 % de défense pendant 1 h (combats de zone et world boss)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10 %</t>
-        </is>
+          <t>2 × Écaille de dragon + 2 × Sang lunaire</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>15</v>
+      </c>
+      <c r="F13" t="n">
+        <v>750</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
+          <t>Élixir de vitalité supérieur</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>elixir_vitalite_sup</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+20 % de PV max pendant 1 h (combats de zone et world boss)</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>2 × Écaille de dragon + 2 × Croc primordial</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Maîtrise</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Potions préparées</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Remise</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Potion offerte</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="n"/>
+      <c r="F16" s="5" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Apprentie</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>0 %</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>0 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Compagne</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>5 %</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>0 %</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="5" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Maîtresse</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>120</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
           <t>Légendaire</t>
         </is>
       </c>
-      <c r="B14" s="5" t="n">
+      <c r="B20" s="5" t="n">
         <v>400</v>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>15 %</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>20 %</t>
         </is>
       </c>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="n"/>
+      <c r="E20" s="5" t="n"/>
+      <c r="F20" s="5" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F14"/>
+  <autoFilter ref="A1:F20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10398,7 +10884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -10545,7 +11031,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Fait apparaître l'élite de le Cimetière abandonné (rang E) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
+          <t>Fait apparaître l'élite du Cimetière abandonné (rang E) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
         </is>
       </c>
     </row>
@@ -10590,19 +11076,19 @@
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Fait apparaître l'élite de le Berceau cataclysmique (rang D) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
+          <t>Fait apparaître l'élite du Berceau cataclysmique (rang D) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>sceau_souffle_e</t>
+          <t>cor_chasse_c</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Sceau du second souffle (rang E)</t>
+          <t>Cor de chasse du Sanctuaire</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -10616,7 +11102,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>700</v>
+        <v>1500</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -10630,24 +11116,24 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>non</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Efface l'attente après un échec à l'épreuve du rang E : tu peux la retenter tout de suite.</t>
+          <t>Fait apparaître l'élite du Sanctuaire primordial (rang C) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>sceau_souffle_d</t>
+          <t>cor_chasse_b</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Sceau du second souffle (rang D)</t>
+          <t>Cor de chasse de l'Éclipse</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -10661,7 +11147,7 @@
         </is>
       </c>
       <c r="E6" s="5" t="n">
-        <v>1500</v>
+        <v>1800</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
@@ -10675,24 +11161,24 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>non</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Efface l'attente après un échec à l'épreuve du rang D : tu peux la retenter tout de suite.</t>
+          <t>Fait apparaître l'élite de l'Éclipse éternelle (rang B) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>sceau_souffle_c</t>
+          <t>cor_chasse_a</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Sceau du second souffle (rang C)</t>
+          <t>Cor de chasse des Cimes</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -10706,7 +11192,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>2300</v>
+        <v>2150</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -10720,24 +11206,24 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>non</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Efface l'attente après un échec à l'épreuve du rang C : tu peux la retenter tout de suite.</t>
+          <t>Fait apparaître l'élite des Cimes des Wyrms (rang A) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>sceau_souffle_b</t>
+          <t>sceau_souffle_e</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Sceau du second souffle (rang B)</t>
+          <t>Sceau du second souffle (rang E)</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -10751,7 +11237,7 @@
         </is>
       </c>
       <c r="E8" s="5" t="n">
-        <v>3000</v>
+        <v>700</v>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
@@ -10770,19 +11256,19 @@
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>Efface l'attente après un échec à l'épreuve du rang B : tu peux la retenter tout de suite.</t>
+          <t>Efface l'attente après un échec à l'épreuve du rang E : tu peux la retenter tout de suite.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>sceau_souffle_a</t>
+          <t>sceau_souffle_d</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Sceau du second souffle (rang A)</t>
+          <t>Sceau du second souffle (rang D)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -10796,7 +11282,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>3800</v>
+        <v>1500</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -10815,19 +11301,19 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Efface l'attente après un échec à l'épreuve du rang A : tu peux la retenter tout de suite.</t>
+          <t>Efface l'attente après un échec à l'épreuve du rang D : tu peux la retenter tout de suite.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>sceau_souffle_s</t>
+          <t>sceau_souffle_c</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Sceau du second souffle (rang S)</t>
+          <t>Sceau du second souffle (rang C)</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -10841,7 +11327,7 @@
         </is>
       </c>
       <c r="E10" s="5" t="n">
-        <v>4500</v>
+        <v>2300</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
@@ -10860,19 +11346,19 @@
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>Efface l'attente après un échec à l'épreuve du rang S : tu peux la retenter tout de suite.</t>
+          <t>Efface l'attente après un échec à l'épreuve du rang C : tu peux la retenter tout de suite.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>sceau_souffle_ss</t>
+          <t>sceau_souffle_b</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Sceau du second souffle (rang SS)</t>
+          <t>Sceau du second souffle (rang B)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -10886,7 +11372,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5300</v>
+        <v>3000</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -10905,19 +11391,19 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Efface l'attente après un échec à l'épreuve du rang SS : tu peux la retenter tout de suite.</t>
+          <t>Efface l'attente après un échec à l'épreuve du rang B : tu peux la retenter tout de suite.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>sceau_souffle_sss</t>
+          <t>sceau_souffle_a</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Sceau du second souffle (rang SSS)</t>
+          <t>Sceau du second souffle (rang A)</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -10931,7 +11417,7 @@
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>6000</v>
+        <v>3800</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
@@ -10950,19 +11436,19 @@
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>Efface l'attente après un échec à l'épreuve du rang SSS : tu peux la retenter tout de suite.</t>
+          <t>Efface l'attente après un échec à l'épreuve du rang A : tu peux la retenter tout de suite.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>parchemin_oubli</t>
+          <t>sceau_souffle_s</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Parchemin d'oubli</t>
+          <t>Sceau du second souffle (rang S)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -10975,39 +11461,39 @@
           <t>common</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" t="n">
+        <v>4500</v>
+      </c>
+      <c r="F13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F13" t="n">
-        <v>150</v>
-      </c>
       <c r="G13" t="inlineStr">
         <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Reprend TOUS tes points de stats (attaque, défense, PV) : replace-les ensuite avec /stats.</t>
+          <t>Efface l'attente après un échec à l'épreuve du rang S : tu peux la retenter tout de suite.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>jeton_arbre</t>
+          <t>sceau_souffle_ss</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Jeton de réinitialisation d'arbre</t>
+          <t>Sceau du second souffle (rang SS)</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -11020,39 +11506,39 @@
           <t>common</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="5" t="n">
+        <v>5300</v>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F14" s="5" t="n">
-        <v>60</v>
-      </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>Réinitialise ton arbre de compétences EN PLUS du reset gratuit de la semaine (à garder pour quand il est déjà pris).</t>
+          <t>Efface l'attente après un échec à l'épreuve du rang SS : tu peux la retenter tout de suite.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>sablier_fidelite</t>
+          <t>sceau_souffle_sss</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Sablier de fidélité</t>
+          <t>Sceau du second souffle (rang SSS)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -11066,7 +11552,7 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -11075,34 +11561,34 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Le premier jour de /daily manqué, ta série n'est pas divisée par deux. Il agit tout seul ; un seul à la fois.</t>
+          <t>Efface l'attente après un échec à l'épreuve du rang SSS : tu peux la retenter tout de suite.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>fond_aube_rosee</t>
+          <t>parchemin_oubli</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Fond — Aube rosée</t>
+          <t>Parchemin d'oubli</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>cosmetic</t>
+          <t>consumable</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -11110,14 +11596,14 @@
           <t>common</t>
         </is>
       </c>
-      <c r="E16" s="5" t="n">
-        <v>2000</v>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="F16" s="5" t="n">
+        <v>150</v>
+      </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
           <t>oui</t>
@@ -11130,24 +11616,24 @@
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>Cosmétique : change le fond de ta bannière /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+          <t>Reprend TOUS tes points de stats (attaque, défense, PV) : replace-les ensuite avec /stats.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>fond_foret_emeraude</t>
+          <t>jeton_arbre</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Fond — Forêt d'émeraude</t>
+          <t>Jeton de réinitialisation d'arbre</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>cosmetic</t>
+          <t>consumable</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -11155,14 +11641,14 @@
           <t>common</t>
         </is>
       </c>
-      <c r="E17" t="n">
-        <v>2000</v>
-      </c>
-      <c r="F17" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="F17" t="n">
+        <v>60</v>
+      </c>
       <c r="G17" t="inlineStr">
         <is>
           <t>oui</t>
@@ -11175,33 +11661,33 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Cosmétique : change le fond de ta bannière /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+          <t>Réinitialise ton arbre de compétences EN PLUS du reset gratuit de la semaine (à garder pour quand il est déjà pris).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>fond_ocean_profond</t>
+          <t>sablier_fidelite</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Fond — Océan profond</t>
+          <t>Sablier de fidélité</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>cosmetic</t>
+          <t>consumable</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>rare</t>
+          <t>common</t>
         </is>
       </c>
       <c r="E18" s="5" t="n">
-        <v>10000</v>
+        <v>2000</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
@@ -11220,19 +11706,19 @@
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>Cosmétique : change le fond de ta bannière /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+          <t>Le premier jour de /daily manqué, ta série n'est pas divisée par deux. Il agit tout seul ; un seul à la fois.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>fond_braises</t>
+          <t>fond_aube_rosee</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Fond — Braises du Berceau</t>
+          <t>Fond — Aube rosée</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -11242,11 +11728,11 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>rare</t>
+          <t>common</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>10000</v>
+        <v>2000</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -11272,12 +11758,12 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>fond_crepuscule_dore</t>
+          <t>fond_foret_emeraude</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Fond — Crépuscule doré</t>
+          <t>Fond — Forêt d'émeraude</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -11287,11 +11773,11 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>epic</t>
+          <t>common</t>
         </is>
       </c>
       <c r="E20" s="5" t="n">
-        <v>40000</v>
+        <v>2000</v>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
@@ -11317,12 +11803,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>fond_aurore_boreale</t>
+          <t>fond_ocean_profond</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Fond — Aurore boréale</t>
+          <t>Fond — Océan profond</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -11332,11 +11818,11 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>legendary</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>150000</v>
+        <v>10000</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -11362,12 +11848,12 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>cadre_argent</t>
+          <t>fond_braises</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Cadre — Argent</t>
+          <t>Fond — Braises du Berceau</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -11377,11 +11863,11 @@
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>common</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="E22" s="5" t="n">
-        <v>2000</v>
+        <v>10000</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
@@ -11400,19 +11886,19 @@
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>Cosmétique : change l'anneau autour de ton avatar sur /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+          <t>Cosmétique : change le fond de ta bannière /profil. Aucun effet en combat. À choisir avec /apparence.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>cadre_jade</t>
+          <t>fond_crepuscule_dore</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Cadre — Jade</t>
+          <t>Fond — Crépuscule doré</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -11422,11 +11908,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>common</t>
+          <t>epic</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>2000</v>
+        <v>40000</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -11445,19 +11931,19 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Cosmétique : change l'anneau autour de ton avatar sur /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+          <t>Cosmétique : change le fond de ta bannière /profil. Aucun effet en combat. À choisir avec /apparence.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>cadre_amethyste</t>
+          <t>fond_aurore_boreale</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Cadre — Améthyste</t>
+          <t>Fond — Aurore boréale</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
@@ -11467,11 +11953,11 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>rare</t>
+          <t>legendary</t>
         </is>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10000</v>
+        <v>150000</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -11490,19 +11976,19 @@
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>Cosmétique : change l'anneau autour de ton avatar sur /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+          <t>Cosmétique : change le fond de ta bannière /profil. Aucun effet en combat. À choisir avec /apparence.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>cadre_or_royal</t>
+          <t>cadre_argent</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Cadre — Or royal</t>
+          <t>Cadre — Argent</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -11512,11 +11998,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>epic</t>
+          <t>common</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>40000</v>
+        <v>2000</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -11542,12 +12028,12 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>cadre_sakura_eternel</t>
+          <t>cadre_jade</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Cadre — Sakura éternel</t>
+          <t>Cadre — Jade</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
@@ -11557,11 +12043,11 @@
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>legendary</t>
+          <t>common</t>
         </is>
       </c>
       <c r="E26" s="5" t="n">
-        <v>150000</v>
+        <v>2000</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
@@ -11587,12 +12073,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>titre_ivoire</t>
+          <t>cadre_amethyste</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Titre — Ivoire</t>
+          <t>Cadre — Améthyste</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -11602,11 +12088,11 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>common</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>2000</v>
+        <v>10000</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -11625,19 +12111,19 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Cosmétique : change la couleur de ton titre sur /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+          <t>Cosmétique : change l'anneau autour de ton avatar sur /profil. Aucun effet en combat. À choisir avec /apparence.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>titre_azur</t>
+          <t>cadre_or_royal</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Titre — Azur</t>
+          <t>Cadre — Or royal</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
@@ -11647,11 +12133,11 @@
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>common</t>
+          <t>epic</t>
         </is>
       </c>
       <c r="E28" s="5" t="n">
-        <v>2000</v>
+        <v>40000</v>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
@@ -11670,19 +12156,19 @@
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>Cosmétique : change la couleur de ton titre sur /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+          <t>Cosmétique : change l'anneau autour de ton avatar sur /profil. Aucun effet en combat. À choisir avec /apparence.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>titre_emeraude</t>
+          <t>cadre_sakura_eternel</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Titre — Émeraude</t>
+          <t>Cadre — Sakura éternel</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -11692,11 +12178,11 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>rare</t>
+          <t>legendary</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>10000</v>
+        <v>150000</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -11715,19 +12201,19 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Cosmétique : change la couleur de ton titre sur /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+          <t>Cosmétique : change l'anneau autour de ton avatar sur /profil. Aucun effet en combat. À choisir avec /apparence.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>titre_rubis</t>
+          <t>titre_ivoire</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Titre — Rubis</t>
+          <t>Titre — Ivoire</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
@@ -11737,11 +12223,11 @@
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>epic</t>
+          <t>common</t>
         </is>
       </c>
       <c r="E30" s="5" t="n">
-        <v>40000</v>
+        <v>2000</v>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
@@ -11767,50 +12253,185 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>titre_azur</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Titre — Azur</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>cosmetic</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Cosmétique : change la couleur de ton titre sur /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>titre_emeraude</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Titre — Émeraude</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>cosmetic</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>Cosmétique : change la couleur de ton titre sur /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>titre_rubis</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Titre — Rubis</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>cosmetic</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>epic</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>40000</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Cosmétique : change la couleur de ton titre sur /profil. Aucun effet en combat. À choisir avec /apparence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
           <t>titre_or_flamboyant</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>Titre — Or flamboyant</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>cosmetic</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D34" s="5" t="inlineStr">
         <is>
           <t>legendary</t>
         </is>
       </c>
-      <c r="E31" t="n">
+      <c r="E34" s="5" t="n">
         <v>150000</v>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F34" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G34" s="5" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="H34" s="5" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="I34" s="5" t="inlineStr">
         <is>
           <t>Cosmétique : change la couleur de ton titre sur /profil. Aucun effet en combat. À choisir avec /apparence.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I31"/>
+  <autoFilter ref="A1:I34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16670,15 +17291,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="29" customWidth="1" min="6" max="6"/>
     <col width="48" customWidth="1" min="7" max="7"/>
     <col width="48" customWidth="1" min="8" max="8"/>
   </cols>
@@ -17595,7 +18216,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>gobelin_superieur / 50</t>
+          <t>gobelin_superieur / 25</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -17605,66 +18226,67 @@
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>50 gobelins supérieurs tués. +5% drop rate sur cette espèce.</t>
+          <t>25 gobelins supérieurs vaincus. +5% drop rate sur cette espèce. (élite de groupe : 25 suffisent)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>mvp_world_boss</t>
+          <t>mort_vivant_slayer</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>MVP des World Boss</t>
+          <t>Pourfendeur de morts-vivants</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>🏆</t>
+          <t>💀</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>non</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>world_boss_mvp</t>
+          <t>kills_family</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>champion_all_stats → value=2</t>
+          <t>mort-vivant / 100</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>damage_bonus_vs_family → target=mort-vivant, value=10
+damage_reduction_from_family → target=mort-vivant, value=10</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Meilleur contributeur du dernier world boss vaincu. +2% sur toutes vos stats. Transmis au MVP du prochain boss.</t>
+          <t>100 morts-vivants vaincus. +10% dégâts infligés et -10% dégâts subis face aux morts-vivants.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>tueur_slime_titan</t>
+          <t>demoniaque_slayer</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Tueur du Titan Visqueux</t>
+          <t>Pourfendeur de démons</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>⚔️</t>
+          <t>😈</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
@@ -17674,39 +18296,40 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>world_boss_kill</t>
+          <t>kills_family</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>slime_titan / 1</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="inlineStr">
-        <is>
-          <t>crit_damage_flat → value=3</t>
+          <t>demoniaque / 100</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>damage_bonus_vs_family → target=demoniaque, value=10
+damage_reduction_from_family → target=demoniaque, value=10</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>A participé à la victoire contre Titan Visqueux. +3 dégâts critiques.</t>
+          <t>100 démons vaincus. +10% dégâts infligés et -10% dégâts subis face aux démons.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>tueur_gobelin_warlord</t>
+          <t>primordial_slayer</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Tueur du Seigneur de Guerre Gobelin</t>
+          <t>Pourfendeur de bêtes primordiales</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>⚔️</t>
+          <t>🐺</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -17716,39 +18339,40 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>world_boss_kill</t>
+          <t>kills_family</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>gobelin_warlord / 1</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>crit_damage_flat → value=3</t>
+          <t>primordial / 100</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>damage_bonus_vs_family → target=primordial, value=10
+damage_reduction_from_family → target=primordial, value=10</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>A participé à la victoire contre Seigneur de Guerre Gobelin. +3 dégâts critiques.</t>
+          <t>100 bêtes primordiales vaincus. +10% dégâts infligés et -10% dégâts subis face aux bêtes primordiales.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>tueur_stone_colossus</t>
+          <t>nocturne_slayer</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Tueur du Colosse de Pierre</t>
+          <t>Pourfendeur des ténèbres</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>⚔️</t>
+          <t>🦇</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
@@ -17758,39 +18382,40 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>world_boss_kill</t>
+          <t>kills_family</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>stone_colossus / 1</t>
-        </is>
-      </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>crit_damage_flat → value=3</t>
+          <t>nocturne / 100</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>damage_bonus_vs_family → target=nocturne, value=10
+damage_reduction_from_family → target=nocturne, value=10</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>A participé à la victoire contre Colosse de Pierre. +3 dégâts critiques.</t>
+          <t>100 créatures nocturnes vaincus. +10% dégâts infligés et -10% dégâts subis face aux créatures nocturnes.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>tueur_shadow_wraith</t>
+          <t>draconique_slayer</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Tueur du Spectre des Ténèbres</t>
+          <t>Pourfendeur de dragons</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>⚔️</t>
+          <t>🐉</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -17800,39 +18425,40 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>world_boss_kill</t>
+          <t>kills_family</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>shadow_wraith / 1</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>crit_damage_flat → value=3</t>
+          <t>draconique / 100</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>damage_bonus_vs_family → target=draconique, value=10
+damage_reduction_from_family → target=draconique, value=10</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>A participé à la victoire contre Spectre des Ténèbres. +3 dégâts critiques.</t>
+          <t>100 dragons vaincus. +10% dégâts infligés et -10% dégâts subis face aux dragons.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>tueur_ancient_dragon</t>
+          <t>abyssal_slayer</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Tueur du Dragon Ancestral</t>
+          <t>Pourfendeur du Néant</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>⚔️</t>
+          <t>🌌</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -17842,57 +18468,2032 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>world_boss_kill</t>
+          <t>kills_family</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>ancient_dragon / 1</t>
-        </is>
-      </c>
-      <c r="G28" s="5" t="inlineStr">
-        <is>
-          <t>crit_damage_flat → value=3</t>
+          <t>abyssal / 100</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>damage_bonus_vs_family → target=abyssal, value=10
+damage_reduction_from_family → target=abyssal, value=10</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>A participé à la victoire contre Dragon Ancestral. +3 dégâts critiques.</t>
+          <t>100 créatures du Néant vaincus. +10% dégâts infligés et -10% dégâts subis face aux créatures du Néant.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>squelette_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Squelette</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>squelette / 50</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=squelette, value=5</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>50 × Squelette vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>zombie_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Zombie</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>zombie / 50</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=zombie, value=5</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>50 × Zombie vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>momie_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Momie</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>momie / 50</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=momie, value=5</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>50 × Momie vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>fantome_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Fantôme</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>fantome / 50</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=fantome, value=5</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>50 × Fantôme vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>gargouille_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Gargouille</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>gargouille / 50</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=gargouille, value=5</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>50 × Gargouille vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>diablotin_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Diablotin</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>diablotin / 50</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=diablotin, value=5</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>50 × Diablotin vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>banshee_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Banshee</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>banshee / 50</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=banshee, value=5</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>50 × Banshee vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>loup_sacre_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Loup sacré</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>loup_sacre / 50</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=loup_sacre, value=5</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>50 × Loup sacré vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>cerf_esprit_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Cerf-esprit</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>cerf_esprit / 50</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=cerf_esprit, value=5</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>50 × Cerf-esprit vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>serpent_des_racines_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Serpent des racines</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>serpent_des_racines / 50</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=serpent_des_racines, value=5</t>
+        </is>
+      </c>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>50 × Serpent des racines vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>demon_cornu_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Démon cornu</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>demon_cornu / 50</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=demon_cornu, value=5</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>50 × Démon cornu vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>ours_colosse_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Ours colosse</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>ours_colosse / 50</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=ours_colosse, value=5</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>50 × Ours colosse vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>liche_maudite_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Liche maudite</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>liche_maudite / 25</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=liche_maudite, value=5</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>25 × Liche maudite vaincus. +5% drop rate sur cette espèce. (élite de groupe : 25 suffisent)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>golem_de_mousse_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Golem de mousse</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>golem_de_mousse / 50</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=golem_de_mousse, value=5</t>
+        </is>
+      </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>50 × Golem de mousse vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>aigle_tempete_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Aigle-tempête</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>aigle_tempete / 25</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=aigle_tempete, value=5</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>25 × Aigle-tempête vaincus. +5% drop rate sur cette espèce. (élite de groupe : 25 suffisent)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>chauve_souris_geante_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Chauve-souris géante</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>chauve_souris_geante / 50</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=chauve_souris_geante, value=5</t>
+        </is>
+      </c>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
+          <t>50 × Chauve-souris géante vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>goule_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Goule</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>goule / 50</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=goule, value=5</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>50 × Goule vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>loup_garou_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Loup-garou</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>loup_garou / 50</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=loup_garou, value=5</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>50 × Loup-garou vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>ogre_demoniaque_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Ogre démoniaque</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>ogre_demoniaque / 50</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=ogre_demoniaque, value=5</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>50 × Ogre démoniaque vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>sorciere_de_sang_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Sorcière de sang</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>sorciere_de_sang / 50</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=sorciere_de_sang, value=5</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t>50 × Sorcière de sang vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>chevalier_de_l_eclipse_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Chevalier de l'éclipse</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>chevalier_de_l_eclipse / 50</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=chevalier_de_l_eclipse, value=5</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>50 × Chevalier de l'éclipse vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>vampire_noble_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Vampire noble</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>vampire_noble / 50</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=vampire_noble, value=5</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
+          <t>50 × Vampire noble vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>comtesse_ecarlate_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Comtesse écarlate</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>comtesse_ecarlate / 25</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=comtesse_ecarlate, value=5</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>25 × Comtesse écarlate vaincus. +5% drop rate sur cette espèce. (élite de groupe : 25 suffisent)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>kobold_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Kobold</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>kobold / 50</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=kobold, value=5</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>50 × Kobold vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>cerbere_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Cerbère</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>cerbere / 50</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=cerbere, value=5</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>50 × Cerbère vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>dragonnet_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Dragonnet</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>dragonnet / 50</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=dragonnet, value=5</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr">
+        <is>
+          <t>50 × Dragonnet vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>drake_de_braise_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Drake de braise</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>drake_de_braise / 50</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=drake_de_braise, value=5</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>50 × Drake de braise vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>wyverne_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Wyverne</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>wyverne / 50</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=wyverne, value=5</t>
+        </is>
+      </c>
+      <c r="H56" s="5" t="inlineStr">
+        <is>
+          <t>50 × Wyverne vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>dragon_de_givre_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Dragon de givre</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>dragon_de_givre / 50</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=dragon_de_givre, value=5</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>50 × Dragon de givre vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>succube_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Succube</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>succube / 50</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=succube, value=5</t>
+        </is>
+      </c>
+      <c r="H58" s="5" t="inlineStr">
+        <is>
+          <t>50 × Succube vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>gardien_draconique_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Gardien draconique</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>gardien_draconique / 50</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=gardien_draconique, value=5</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>50 × Gardien draconique vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>dragon_ancien_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Dragon ancien</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>dragon_ancien / 25</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=dragon_ancien, value=5</t>
+        </is>
+      </c>
+      <c r="H60" s="5" t="inlineStr">
+        <is>
+          <t>25 × Dragon ancien vaincus. +5% drop rate sur cette espèce. (élite de groupe : 25 suffisent)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>rejeton_du_neant_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Rejeton du néant</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>rejeton_du_neant / 50</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=rejeton_du_neant, value=5</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>50 × Rejeton du néant vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>oeil_errant_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Œil errant</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F62" s="5" t="inlineStr">
+        <is>
+          <t>oeil_errant / 50</t>
+        </is>
+      </c>
+      <c r="G62" s="5" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=oeil_errant, value=5</t>
+        </is>
+      </c>
+      <c r="H62" s="5" t="inlineStr">
+        <is>
+          <t>50 × Œil errant vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>ange_dechu_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Ange déchu</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>ange_dechu / 50</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=ange_dechu, value=5</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>50 × Ange déchu vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>devoreur_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Dévoreur</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>devoreur / 50</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=devoreur, value=5</t>
+        </is>
+      </c>
+      <c r="H64" s="5" t="inlineStr">
+        <is>
+          <t>50 × Dévoreur vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>heraut_du_vide_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Héraut du vide</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>heraut_du_vide / 50</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=heraut_du_vide, value=5</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>50 × Héraut du vide vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>kraken_astral_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Kraken astral</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>kraken_astral / 50</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=kraken_astral, value=5</t>
+        </is>
+      </c>
+      <c r="H66" s="5" t="inlineStr">
+        <is>
+          <t>50 × Kraken astral vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>seraphin_brise_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Séraphin brisé</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>seraphin_brise / 50</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=seraphin_brise, value=5</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>50 × Séraphin brisé vaincus. +5% drop rate sur cette espèce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>archidemon_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Archidémon</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>archidemon / 25</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=archidemon, value=5</t>
+        </is>
+      </c>
+      <c r="H68" s="5" t="inlineStr">
+        <is>
+          <t>25 × Archidémon vaincus. +5% drop rate sur cette espèce. (élite de groupe : 25 suffisent)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>avatar_du_neant_chasseur_legendaire</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Chasseur Légendaire — Avatar du Néant</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>🏹</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>kills_mob</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>avatar_du_neant / 25</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>drop_rate_bonus_vs_mob → target=avatar_du_neant, value=5</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>25 × Avatar du Néant vaincus. +5% drop rate sur cette espèce. (élite de groupe : 25 suffisent)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>mvp_world_boss</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>MVP des World Boss</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>🏆</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>world_boss_mvp</t>
+        </is>
+      </c>
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G70" s="5" t="inlineStr">
+        <is>
+          <t>champion_all_stats → value=2</t>
+        </is>
+      </c>
+      <c r="H70" s="5" t="inlineStr">
+        <is>
+          <t>Meilleur contributeur du dernier world boss vaincu. +2% sur toutes vos stats. Transmis au MVP du prochain boss.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>tueur_slime_titan</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Tueur du Titan Visqueux</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>⚔️</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>world_boss_kill</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>slime_titan / 1</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>crit_damage_flat → value=3</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>A participé à la victoire contre Titan Visqueux. +3 dégâts critiques.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>tueur_gobelin_warlord</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>Tueur du Seigneur de Guerre Gobelin</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>⚔️</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>world_boss_kill</t>
+        </is>
+      </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>gobelin_warlord / 1</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>crit_damage_flat → value=3</t>
+        </is>
+      </c>
+      <c r="H72" s="5" t="inlineStr">
+        <is>
+          <t>A participé à la victoire contre Seigneur de Guerre Gobelin. +3 dégâts critiques.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>tueur_stone_colossus</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Tueur du Colosse de Pierre</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>⚔️</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>world_boss_kill</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>stone_colossus / 1</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>crit_damage_flat → value=3</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>A participé à la victoire contre Colosse de Pierre. +3 dégâts critiques.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>tueur_shadow_wraith</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>Tueur du Spectre des Ténèbres</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>⚔️</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>world_boss_kill</t>
+        </is>
+      </c>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>shadow_wraith / 1</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>crit_damage_flat → value=3</t>
+        </is>
+      </c>
+      <c r="H74" s="5" t="inlineStr">
+        <is>
+          <t>A participé à la victoire contre Spectre des Ténèbres. +3 dégâts critiques.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>tueur_ancient_dragon</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Tueur du Dragon Ancestral</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>⚔️</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>world_boss_kill</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>ancient_dragon / 1</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>crit_damage_flat → value=3</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>A participé à la victoire contre Dragon Ancestral. +3 dégâts critiques.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
           <t>ma_survie_avant_tout</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B76" s="5" t="inlineStr">
         <is>
           <t>Ma survie avant tout</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C76" s="5" t="inlineStr">
         <is>
           <t>🛡️</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D76" s="5" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E76" s="5" t="inlineStr">
         <is>
           <t>event</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F76" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G29" s="8" t="inlineStr">
+      <c r="G76" s="7" t="inlineStr">
         <is>
           <t>dodge_flat → value=1
 speed_flat → value=1
@@ -17900,14 +20501,14 @@
 hp_max_flat → value=200</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="H76" s="5" t="inlineStr">
         <is>
           <t>A ignoré une « petite fille » qui s'est révélée être un monstre déguisé — l'instinct de survie récompensé. Esquive +1%, Vitesse +1, Défense +10, PV max +200.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H29"/>
+  <autoFilter ref="A1:H76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(zones): ouverture des zones C, B et A
Sanctuaire primordial (C), Éclipse éternelle (B) et Cimes des Wyrms (A)
passent dans les zones ouvertes avec leurs salons. Familles existantes
recalées dans leur tranche, élites recalibrées sur le trio de leur
nouveau niveau, cors C/B/A actifs et prix de tous les cors recalculés.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sakura_content.xlsx
+++ b/docs/sakura_content.xlsx
@@ -511,7 +511,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 2026-10-26 13:23 UTC</t>
+          <t>Généré le 2026-10-27 07:50 UTC</t>
         </is>
       </c>
     </row>
@@ -5608,13 +5608,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>154</v>
+        <v>121</v>
       </c>
       <c r="E3" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G3" t="n">
         <v>5</v>
@@ -5632,10 +5632,10 @@
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="M3" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="N3" t="n">
         <v>40</v>
@@ -5677,13 +5677,13 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>198</v>
+        <v>143</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G4" s="5" t="n">
         <v>5</v>
@@ -5701,10 +5701,10 @@
         <v>0</v>
       </c>
       <c r="L4" s="5" t="n">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="N4" s="5" t="n">
         <v>30</v>
@@ -5732,27 +5732,27 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>squelette</t>
+          <t>gobelin_chaman</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Squelette</t>
+          <t>Gobelin Chaman</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>mort-vivant</t>
+          <t>gobelin</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>231</v>
+        <v>141</v>
       </c>
       <c r="E5" t="n">
         <v>26</v>
       </c>
       <c r="F5" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G5" t="n">
         <v>5</v>
@@ -5770,13 +5770,13 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>88</v>
+        <v>50</v>
       </c>
       <c r="M5" t="n">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="N5" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="O5" s="6">
         <f>ROUND((E5*(1+(H5/100)*MAX(0,I5-100)/100)*(1+G5/100))*((D5+F5*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J5/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -5789,24 +5789,24 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>squelette.png</t>
+          <t>gobelin_chaman.png</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>Un pantin d'os réanimé. Le premier pas dans le royaume des morts.</t>
+          <t>Une créature intelligente.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>gobelin_chaman</t>
+          <t>gobelin_ballon</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Gobelin Chaman</t>
+          <t>Gobelin Ballon</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -5815,13 +5815,13 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G6" s="5" t="n">
         <v>5</v>
@@ -5839,13 +5839,13 @@
         <v>0</v>
       </c>
       <c r="L6" s="5" t="n">
-        <v>94</v>
+        <v>62</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="N6" s="5" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="O6" s="6">
         <f>ROUND((E6*(1+(H6/100)*MAX(0,I6-100)/100)*(1+G6/100))*((D6+F6*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J6/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -5858,39 +5858,39 @@
       <c r="Q6" s="5" t="inlineStr"/>
       <c r="R6" s="5" t="inlineStr">
         <is>
-          <t>gobelin_chaman.png</t>
+          <t>gobelin_ballon.png</t>
         </is>
       </c>
       <c r="S6" s="5" t="inlineStr">
         <is>
-          <t>Une créature intelligente.</t>
+          <t>Un groupe de créatures inventives.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>zombie</t>
+          <t>gobelin_geant</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Zombie</t>
+          <t>Gobelin Géant</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>mort-vivant</t>
+          <t>gobelin</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>248</v>
+        <v>188</v>
       </c>
       <c r="E7" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F7" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G7" t="n">
         <v>5</v>
@@ -5908,10 +5908,10 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>112</v>
+        <v>75</v>
       </c>
       <c r="M7" t="n">
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="N7" t="n">
         <v>20</v>
@@ -5927,24 +5927,24 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>zombie.png</t>
+          <t>gobelin_geant.png</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Une carcasse putride et lente, mais coriace.</t>
+          <t>Une créature imposante.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>gobelin_ballon</t>
+          <t>gobelin_runique</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Gobelin Ballon</t>
+          <t>Gobelin Runique</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -5953,13 +5953,13 @@
         </is>
       </c>
       <c r="D8" s="5" t="n">
-        <v>286</v>
+        <v>194</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="G8" s="5" t="n">
         <v>5</v>
@@ -5977,10 +5977,10 @@
         <v>0</v>
       </c>
       <c r="L8" s="5" t="n">
-        <v>119</v>
+        <v>94</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="N8" s="5" t="n">
         <v>20</v>
@@ -5996,24 +5996,24 @@
       <c r="Q8" s="5" t="inlineStr"/>
       <c r="R8" s="5" t="inlineStr">
         <is>
-          <t>gobelin_ballon.png</t>
+          <t>gobelin_runique.png</t>
         </is>
       </c>
       <c r="S8" s="5" t="inlineStr">
         <is>
-          <t>Un groupe de créatures inventives.</t>
+          <t>Une créature mystérieuse.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>gobelin_geant</t>
+          <t>gobelin_assassin</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Gobelin Géant</t>
+          <t>Gobelin Assassin</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -6022,22 +6022,22 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>287</v>
+        <v>158</v>
       </c>
       <c r="E9" t="n">
         <v>28</v>
       </c>
       <c r="F9" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="G9" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I9" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -6046,13 +6046,13 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>144</v>
+        <v>106</v>
       </c>
       <c r="M9" t="n">
-        <v>69</v>
+        <v>51</v>
       </c>
       <c r="N9" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="O9" s="6">
         <f>ROUND((E9*(1+(H9/100)*MAX(0,I9-100)/100)*(1+G9/100))*((D9+F9*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J9/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -6065,42 +6065,42 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>gobelin_geant.png</t>
+          <t>gobelin_assassin.png</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Une créature imposante.</t>
+          <t>Une créature discrète.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>momie</t>
+          <t>gobelin_superieur</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Momie</t>
+          <t>Gobelin Supérieur</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>mort-vivant</t>
+          <t>gobelin</t>
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>330</v>
+        <v>286</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>41</v>
+        <v>143</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H10" s="5" t="n">
         <v>0</v>
@@ -6115,10 +6115,10 @@
         <v>0</v>
       </c>
       <c r="L10" s="5" t="n">
-        <v>150</v>
+        <v>375</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>72</v>
+        <v>180</v>
       </c>
       <c r="N10" s="5" t="n">
         <v>10</v>
@@ -6134,39 +6134,39 @@
       <c r="Q10" s="5" t="inlineStr"/>
       <c r="R10" s="5" t="inlineStr">
         <is>
-          <t>momie.png</t>
+          <t>gobelin_superieur.png</t>
         </is>
       </c>
       <c r="S10" s="5" t="inlineStr">
         <is>
-          <t>Un corps embaumé aux bandelettes maudites, quasi increvable.</t>
+          <t>Une créature supérieure.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>gobelin_runique</t>
+          <t>squelette</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Gobelin Runique</t>
+          <t>Squelette</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>gobelin</t>
+          <t>mort-vivant</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="E11" t="n">
-        <v>69</v>
+        <v>37</v>
       </c>
       <c r="F11" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="G11" t="n">
         <v>6</v>
@@ -6184,13 +6184,13 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>169</v>
+        <v>131</v>
       </c>
       <c r="M11" t="n">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="N11" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="O11" s="6">
         <f>ROUND((E11*(1+(H11/100)*MAX(0,I11-100)/100)*(1+G11/100))*((D11+F11*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J11/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -6203,24 +6203,24 @@
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>gobelin_runique.png</t>
+          <t>squelette.png</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Une créature mystérieuse.</t>
+          <t>Un pantin d'os réanimé. Le premier pas dans le royaume des morts.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>fantome</t>
+          <t>zombie</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Fantôme</t>
+          <t>Zombie</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -6229,37 +6229,37 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>231</v>
+        <v>287</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="H12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="J12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="5" t="n">
+        <v>144</v>
+      </c>
+      <c r="M12" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="N12" s="5" t="n">
         <v>20</v>
-      </c>
-      <c r="I12" s="5" t="n">
-        <v>150</v>
-      </c>
-      <c r="J12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" s="5" t="n">
-        <v>188</v>
-      </c>
-      <c r="M12" s="5" t="n">
-        <v>90</v>
-      </c>
-      <c r="N12" s="5" t="n">
-        <v>15</v>
       </c>
       <c r="O12" s="6">
         <f>ROUND((E12*(1+(H12/100)*MAX(0,I12-100)/100)*(1+G12/100))*((D12+F12*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J12/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -6272,48 +6272,48 @@
       <c r="Q12" s="5" t="inlineStr"/>
       <c r="R12" s="5" t="inlineStr">
         <is>
-          <t>fantome.png</t>
+          <t>zombie.png</t>
         </is>
       </c>
       <c r="S12" s="5" t="inlineStr">
         <is>
-          <t>Une âme errante insaisissable qui glisse entre les coups.</t>
+          <t>Une carcasse putride et lente, mais coriace.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>gobelin_assassin</t>
+          <t>momie</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Gobelin Assassin</t>
+          <t>Momie</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>gobelin</t>
+          <t>mort-vivant</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>238</v>
+        <v>341</v>
       </c>
       <c r="E13" t="n">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="F13" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G13" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="H13" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -6322,10 +6322,10 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>194</v>
+        <v>156</v>
       </c>
       <c r="M13" t="n">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="N13" t="n">
         <v>10</v>
@@ -6341,48 +6341,48 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>gobelin_assassin.png</t>
+          <t>momie.png</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>Une créature discrète.</t>
+          <t>Un corps embaumé aux bandelettes maudites, quasi increvable.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>gobelin_superieur</t>
+          <t>fantome</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Gobelin Supérieur</t>
+          <t>Fantôme</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>gobelin</t>
+          <t>mort-vivant</t>
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>1320</v>
+        <v>218</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>178</v>
+        <v>41</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0</v>
@@ -6391,13 +6391,13 @@
         <v>0</v>
       </c>
       <c r="L14" s="5" t="n">
-        <v>656</v>
+        <v>169</v>
       </c>
       <c r="M14" s="5" t="n">
-        <v>315</v>
+        <v>81</v>
       </c>
       <c r="N14" s="5" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="O14" s="6">
         <f>ROUND((E14*(1+(H14/100)*MAX(0,I14-100)/100)*(1+G14/100))*((D14+F14*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J14/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -6410,12 +6410,12 @@
       <c r="Q14" s="5" t="inlineStr"/>
       <c r="R14" s="5" t="inlineStr">
         <is>
-          <t>gobelin_superieur.png</t>
+          <t>fantome.png</t>
         </is>
       </c>
       <c r="S14" s="5" t="inlineStr">
         <is>
-          <t>Une créature supérieure.</t>
+          <t>Une âme errante insaisissable qui glisse entre les coups.</t>
         </is>
       </c>
     </row>
@@ -6436,13 +6436,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>426</v>
+        <v>337</v>
       </c>
       <c r="E15" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="F15" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="G15" t="n">
         <v>6</v>
@@ -6460,10 +6460,10 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>238</v>
+        <v>181</v>
       </c>
       <c r="M15" t="n">
-        <v>114</v>
+        <v>87</v>
       </c>
       <c r="N15" t="n">
         <v>7</v>
@@ -6491,36 +6491,36 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>diablotin</t>
+          <t>banshee</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Diablotin</t>
+          <t>Banshee</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>demoniaque</t>
+          <t>mort-vivant</t>
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>323</v>
+        <v>317</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>0</v>
@@ -6529,13 +6529,13 @@
         <v>0</v>
       </c>
       <c r="L16" s="5" t="n">
-        <v>275</v>
+        <v>194</v>
       </c>
       <c r="M16" s="5" t="n">
-        <v>132</v>
+        <v>93</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="O16" s="6">
         <f>ROUND((E16*(1+(H16/100)*MAX(0,I16-100)/100)*(1+G16/100))*((D16+F16*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J16/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -6548,24 +6548,24 @@
       <c r="Q16" s="5" t="inlineStr"/>
       <c r="R16" s="5" t="inlineStr">
         <is>
-          <t>diablotin.png</t>
+          <t>banshee.png</t>
         </is>
       </c>
       <c r="S16" s="5" t="inlineStr">
         <is>
-          <t>Petit démon espiègle et véloce, tout juste éclos du Berceau.</t>
+          <t>Un spectre hurlant dont le cri glaçant transperce l'âme.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>banshee</t>
+          <t>liche_maudite</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Banshee</t>
+          <t>Liche maudite</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -6574,16 +6574,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>440</v>
+        <v>4013</v>
       </c>
       <c r="E17" t="n">
-        <v>117</v>
+        <v>63</v>
       </c>
       <c r="F17" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G17" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -6598,13 +6598,13 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>281</v>
+        <v>619</v>
       </c>
       <c r="M17" t="n">
-        <v>135</v>
+        <v>297</v>
       </c>
       <c r="N17" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O17" s="6">
         <f>ROUND((E17*(1+(H17/100)*MAX(0,I17-100)/100)*(1+G17/100))*((D17+F17*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J17/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -6617,42 +6617,42 @@
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>banshee.png</t>
+          <t>liche_maudite.png</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>Un spectre hurlant dont le cri glaçant transperce l'âme.</t>
+          <t>Un sorcier mort-vivant dont la magie noire dévaste.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>loup_sacre</t>
+          <t>diablotin</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Loup sacré</t>
+          <t>Diablotin</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>primordial</t>
+          <t>demoniaque</t>
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>337</v>
+        <v>257</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>72</v>
+        <v>52</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H18" s="5" t="n">
         <v>20</v>
@@ -6667,10 +6667,10 @@
         <v>0</v>
       </c>
       <c r="L18" s="5" t="n">
-        <v>288</v>
+        <v>212</v>
       </c>
       <c r="M18" s="5" t="n">
-        <v>138</v>
+        <v>102</v>
       </c>
       <c r="N18" s="5" t="n">
         <v>40</v>
@@ -6684,40 +6684,44 @@
         <v/>
       </c>
       <c r="Q18" s="5" t="inlineStr"/>
-      <c r="R18" s="5" t="inlineStr"/>
+      <c r="R18" s="5" t="inlineStr">
+        <is>
+          <t>diablotin.png</t>
+        </is>
+      </c>
       <c r="S18" s="5" t="inlineStr">
         <is>
-          <t>Gardien à la fourrure d'argent ; il chasse en meute depuis l'aube des temps.</t>
+          <t>Petit démon espiègle et véloce, tout juste éclos du Berceau.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>cerf_esprit</t>
+          <t>demon_cornu</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Cerf-esprit</t>
+          <t>Démon cornu</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>primordial</t>
+          <t>demoniaque</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>583</v>
+        <v>451</v>
       </c>
       <c r="E19" t="n">
-        <v>85</v>
+        <v>61</v>
       </c>
       <c r="F19" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="G19" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
@@ -6732,10 +6736,10 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>300</v>
+        <v>225</v>
       </c>
       <c r="M19" t="n">
-        <v>144</v>
+        <v>108</v>
       </c>
       <c r="N19" t="n">
         <v>30</v>
@@ -6749,61 +6753,65 @@
         <v/>
       </c>
       <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>demon_cornu.png</t>
+        </is>
+      </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>Un cerf translucide ; la forêt se tait sur son passage.</t>
+          <t>Fantassin cornu des légions infernales, brutal et sans pitié.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>serpent_des_racines</t>
+          <t>ogre_demoniaque</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Serpent des racines</t>
+          <t>Ogre démoniaque</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>primordial</t>
+          <t>demoniaque</t>
         </is>
       </c>
       <c r="D20" s="5" t="n">
-        <v>363</v>
+        <v>378</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="F20" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="J20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="5" t="n">
+        <v>238</v>
+      </c>
+      <c r="M20" s="5" t="n">
+        <v>114</v>
+      </c>
+      <c r="N20" s="5" t="n">
         <v>20</v>
-      </c>
-      <c r="G20" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="H20" s="5" t="n">
-        <v>20</v>
-      </c>
-      <c r="I20" s="5" t="n">
-        <v>150</v>
-      </c>
-      <c r="J20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" s="5" t="n">
-        <v>312</v>
-      </c>
-      <c r="M20" s="5" t="n">
-        <v>150</v>
-      </c>
-      <c r="N20" s="5" t="n">
-        <v>25</v>
       </c>
       <c r="O20" s="6">
         <f>ROUND((E20*(1+(H20/100)*MAX(0,I20-100)/100)*(1+G20/100))*((D20+F20*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J20/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -6814,22 +6822,26 @@
         <v/>
       </c>
       <c r="Q20" s="5" t="inlineStr"/>
-      <c r="R20" s="5" t="inlineStr"/>
+      <c r="R20" s="5" t="inlineStr">
+        <is>
+          <t>ogre_demoniaque.png</t>
+        </is>
+      </c>
       <c r="S20" s="5" t="inlineStr">
         <is>
-          <t>Il dort sous les racines et frappe d'un venin sylvestre.</t>
+          <t>Masse de muscles corrompue qui écrase tout sur son passage.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>demon_cornu</t>
+          <t>cerbere</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Démon cornu</t>
+          <t>Cerbère</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -6838,16 +6850,16 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>638</v>
+        <v>495</v>
       </c>
       <c r="E21" t="n">
-        <v>93</v>
+        <v>68</v>
       </c>
       <c r="F21" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="G21" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
@@ -6862,13 +6874,13 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>325</v>
+        <v>250</v>
       </c>
       <c r="M21" t="n">
-        <v>156</v>
+        <v>120</v>
       </c>
       <c r="N21" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="O21" s="6">
         <f>ROUND((E21*(1+(H21/100)*MAX(0,I21-100)/100)*(1+G21/100))*((D21+F21*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J21/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -6881,39 +6893,39 @@
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
-          <t>demon_cornu.png</t>
+          <t>cerbere.png</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>Fantassin cornu des légions infernales, brutal et sans pitié.</t>
+          <t>Molosse à trois têtes gardant les portes de l'abîme.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>ours_colosse</t>
+          <t>succube</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Ours colosse</t>
+          <t>Succube</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>primordial</t>
+          <t>demoniaque</t>
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>510</v>
+        <v>414</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>140</v>
+        <v>109</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G22" s="5" t="n">
         <v>7</v>
@@ -6931,13 +6943,13 @@
         <v>0</v>
       </c>
       <c r="L22" s="5" t="n">
-        <v>325</v>
+        <v>262</v>
       </c>
       <c r="M22" s="5" t="n">
-        <v>156</v>
+        <v>126</v>
       </c>
       <c r="N22" s="5" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="O22" s="6">
         <f>ROUND((E22*(1+(H22/100)*MAX(0,I22-100)/100)*(1+G22/100))*((D22+F22*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J22/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -6948,37 +6960,41 @@
         <v/>
       </c>
       <c r="Q22" s="5" t="inlineStr"/>
-      <c r="R22" s="5" t="inlineStr"/>
+      <c r="R22" s="5" t="inlineStr">
+        <is>
+          <t>succube.png</t>
+        </is>
+      </c>
       <c r="S22" s="5" t="inlineStr">
         <is>
-          <t>Ses griffes fendent la pierre comme l'armure.</t>
+          <t>Démone envoûtante qui draine la vie de ses proies.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>liche_maudite</t>
+          <t>ange_dechu</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Liche maudite</t>
+          <t>Ange déchu</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>mort-vivant</t>
+          <t>demoniaque</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>9504</v>
+        <v>539</v>
       </c>
       <c r="E23" t="n">
-        <v>146</v>
+        <v>76</v>
       </c>
       <c r="F23" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="G23" t="n">
         <v>7</v>
@@ -6996,13 +7012,13 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>1012</v>
+        <v>275</v>
       </c>
       <c r="M23" t="n">
-        <v>486</v>
+        <v>132</v>
       </c>
       <c r="N23" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="O23" s="6">
         <f>ROUND((E23*(1+(H23/100)*MAX(0,I23-100)/100)*(1+G23/100))*((D23+F23*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J23/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -7015,39 +7031,39 @@
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
-          <t>liche_maudite.png</t>
+          <t>ange_dechu.png</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>Un sorcier mort-vivant dont la magie noire dévaste.</t>
+          <t>Ancien séraphin banni ; sa lumière s'est muée en fureur.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>golem_de_mousse</t>
+          <t>archidemon</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Golem de mousse</t>
+          <t>Archidémon</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>primordial</t>
+          <t>demoniaque</t>
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>594</v>
+        <v>2970</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="F24" s="5" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="G24" s="5" t="n">
         <v>7</v>
@@ -7065,13 +7081,13 @@
         <v>0</v>
       </c>
       <c r="L24" s="5" t="n">
-        <v>338</v>
+        <v>844</v>
       </c>
       <c r="M24" s="5" t="n">
-        <v>162</v>
+        <v>405</v>
       </c>
       <c r="N24" s="5" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="O24" s="6">
         <f>ROUND((E24*(1+(H24/100)*MAX(0,I24-100)/100)*(1+G24/100))*((D24+F24*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J24/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -7082,22 +7098,26 @@
         <v/>
       </c>
       <c r="Q24" s="5" t="inlineStr"/>
-      <c r="R24" s="5" t="inlineStr"/>
+      <c r="R24" s="5" t="inlineStr">
+        <is>
+          <t>archidemon.png</t>
+        </is>
+      </c>
       <c r="S24" s="5" t="inlineStr">
         <is>
-          <t>Un rocher couvert de mousse qui repousse plus vite qu'on ne l'arrache.</t>
+          <t>Seigneur des enfers, apogée de la corruption du Berceau.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>aigle_tempete</t>
+          <t>loup_sacre</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Aigle-tempête</t>
+          <t>Loup sacré</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -7106,13 +7126,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>3274</v>
+        <v>337</v>
       </c>
       <c r="E25" t="n">
-        <v>138</v>
+        <v>72</v>
       </c>
       <c r="F25" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G25" t="n">
         <v>13</v>
@@ -7130,13 +7150,13 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>1050</v>
+        <v>288</v>
       </c>
       <c r="M25" t="n">
-        <v>504</v>
+        <v>138</v>
       </c>
       <c r="N25" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="O25" s="6">
         <f>ROUND((E25*(1+(H25/100)*MAX(0,I25-100)/100)*(1+G25/100))*((D25+F25*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J25/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -7150,43 +7170,43 @@
       <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr">
         <is>
-          <t>Chacun de ses battements d'ailes soulève une bourrasque.</t>
+          <t>Gardien à la fourrure d'argent ; il chasse en meute depuis l'aube des temps.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>chauve_souris_geante</t>
+          <t>cerf_esprit</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Chauve-souris géante</t>
+          <t>Cerf-esprit</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>nocturne</t>
+          <t>primordial</t>
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>416</v>
+        <v>583</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="F26" s="5" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="J26" s="5" t="n">
         <v>0</v>
@@ -7195,13 +7215,13 @@
         <v>0</v>
       </c>
       <c r="L26" s="5" t="n">
-        <v>356</v>
+        <v>300</v>
       </c>
       <c r="M26" s="5" t="n">
-        <v>171</v>
+        <v>144</v>
       </c>
       <c r="N26" s="5" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O26" s="6">
         <f>ROUND((E26*(1+(H26/100)*MAX(0,I26-100)/100)*(1+G26/100))*((D26+F26*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J26/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -7215,43 +7235,43 @@
       <c r="R26" s="5" t="inlineStr"/>
       <c r="S26" s="5" t="inlineStr">
         <is>
-          <t>Elle surgit de l'éclipse par nuées entières.</t>
+          <t>Un cerf translucide ; la forêt se tait sur son passage.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>goule</t>
+          <t>serpent_des_racines</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Goule</t>
+          <t>Serpent des racines</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>nocturne</t>
+          <t>primordial</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>715</v>
+        <v>363</v>
       </c>
       <c r="E27" t="n">
-        <v>107</v>
+        <v>80</v>
       </c>
       <c r="F27" t="n">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="G27" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="H27" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I27" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -7260,13 +7280,13 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>362</v>
+        <v>312</v>
       </c>
       <c r="M27" t="n">
-        <v>174</v>
+        <v>150</v>
       </c>
       <c r="N27" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="O27" s="6">
         <f>ROUND((E27*(1+(H27/100)*MAX(0,I27-100)/100)*(1+G27/100))*((D27+F27*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J27/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -7280,37 +7300,37 @@
       <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr">
         <is>
-          <t>Elle rôde entre les tombes, affamée de chair fraîche.</t>
+          <t>Il dort sous les racines et frappe d'un venin sylvestre.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>loup_garou</t>
+          <t>ours_colosse</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Loup-garou</t>
+          <t>Ours colosse</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>nocturne</t>
+          <t>primordial</t>
         </is>
       </c>
       <c r="D28" s="5" t="n">
-        <v>590</v>
+        <v>510</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>168</v>
+        <v>140</v>
       </c>
       <c r="F28" s="5" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G28" s="5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H28" s="5" t="n">
         <v>0</v>
@@ -7325,13 +7345,13 @@
         <v>0</v>
       </c>
       <c r="L28" s="5" t="n">
-        <v>375</v>
+        <v>325</v>
       </c>
       <c r="M28" s="5" t="n">
-        <v>180</v>
+        <v>156</v>
       </c>
       <c r="N28" s="5" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="O28" s="6">
         <f>ROUND((E28*(1+(H28/100)*MAX(0,I28-100)/100)*(1+G28/100))*((D28+F28*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J28/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -7345,37 +7365,37 @@
       <c r="R28" s="5" t="inlineStr"/>
       <c r="S28" s="5" t="inlineStr">
         <is>
-          <t>Sous l'éclipse, la bête l'emporte sur l'homme — et sa rage grandit avec ses blessures.</t>
+          <t>Ses griffes fendent la pierre comme l'armure.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ogre_demoniaque</t>
+          <t>golem_de_mousse</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Ogre démoniaque</t>
+          <t>Golem de mousse</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>demoniaque</t>
+          <t>primordial</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>607</v>
+        <v>594</v>
       </c>
       <c r="E29" t="n">
-        <v>176</v>
+        <v>68</v>
       </c>
       <c r="F29" t="n">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="G29" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
@@ -7390,13 +7410,13 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>388</v>
+        <v>338</v>
       </c>
       <c r="M29" t="n">
-        <v>186</v>
+        <v>162</v>
       </c>
       <c r="N29" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="O29" s="6">
         <f>ROUND((E29*(1+(H29/100)*MAX(0,I29-100)/100)*(1+G29/100))*((D29+F29*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J29/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -7407,50 +7427,46 @@
         <v/>
       </c>
       <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>ogre_demoniaque.png</t>
-        </is>
-      </c>
+      <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr">
         <is>
-          <t>Masse de muscles corrompue qui écrase tout sur son passage.</t>
+          <t>Un rocher couvert de mousse qui repousse plus vite qu'on ne l'arrache.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>sorciere_de_sang</t>
+          <t>aigle_tempete</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Sorcière de sang</t>
+          <t>Aigle-tempête</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>nocturne</t>
+          <t>primordial</t>
         </is>
       </c>
       <c r="D30" s="5" t="n">
-        <v>607</v>
+        <v>3274</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>176</v>
+        <v>138</v>
       </c>
       <c r="F30" s="5" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="G30" s="5" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="J30" s="5" t="n">
         <v>0</v>
@@ -7459,13 +7475,13 @@
         <v>0</v>
       </c>
       <c r="L30" s="5" t="n">
-        <v>388</v>
+        <v>1050</v>
       </c>
       <c r="M30" s="5" t="n">
-        <v>186</v>
+        <v>504</v>
       </c>
       <c r="N30" s="5" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="O30" s="6">
         <f>ROUND((E30*(1+(H30/100)*MAX(0,I30-100)/100)*(1+G30/100))*((D30+F30*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J30/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -7479,19 +7495,19 @@
       <c r="R30" s="5" t="inlineStr"/>
       <c r="S30" s="5" t="inlineStr">
         <is>
-          <t>Elle appelle ses familiers d'un murmure.</t>
+          <t>Chacun de ses battements d'ailes soulève une bourrasque.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>chevalier_de_l_eclipse</t>
+          <t>chauve_souris_geante</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Chevalier de l'éclipse</t>
+          <t>Chauve-souris géante</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -7500,22 +7516,22 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>713</v>
+        <v>416</v>
       </c>
       <c r="E31" t="n">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="F31" t="n">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="G31" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I31" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -7524,13 +7540,13 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>400</v>
+        <v>356</v>
       </c>
       <c r="M31" t="n">
-        <v>192</v>
+        <v>171</v>
       </c>
       <c r="N31" t="n">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="O31" s="6">
         <f>ROUND((E31*(1+(H31/100)*MAX(0,I31-100)/100)*(1+G31/100))*((D31+F31*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J31/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -7544,19 +7560,19 @@
       <c r="R31" t="inlineStr"/>
       <c r="S31" t="inlineStr">
         <is>
-          <t>Son armure noire rend chaque coup à celui qui l'a porté.</t>
+          <t>Elle surgit de l'éclipse par nuées entières.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>vampire_noble</t>
+          <t>goule</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Vampire noble</t>
+          <t>Goule</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
@@ -7565,16 +7581,16 @@
         </is>
       </c>
       <c r="D32" s="5" t="n">
-        <v>814</v>
+        <v>715</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>126</v>
+        <v>107</v>
       </c>
       <c r="F32" s="5" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="G32" s="5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H32" s="5" t="n">
         <v>0</v>
@@ -7589,13 +7605,13 @@
         <v>0</v>
       </c>
       <c r="L32" s="5" t="n">
-        <v>412</v>
+        <v>362</v>
       </c>
       <c r="M32" s="5" t="n">
-        <v>198</v>
+        <v>174</v>
       </c>
       <c r="N32" s="5" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="O32" s="6">
         <f>ROUND((E32*(1+(H32/100)*MAX(0,I32-100)/100)*(1+G32/100))*((D32+F32*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J32/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -7609,19 +7625,19 @@
       <c r="R32" s="5" t="inlineStr"/>
       <c r="S32" s="5" t="inlineStr">
         <is>
-          <t>Il boit la vie de ses adversaires avec élégance.</t>
+          <t>Elle rôde entre les tombes, affamée de chair fraîche.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>comtesse_ecarlate</t>
+          <t>loup_garou</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Comtesse écarlate</t>
+          <t>Loup-garou</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -7630,22 +7646,22 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>8910</v>
+        <v>590</v>
       </c>
       <c r="E33" t="n">
-        <v>344</v>
+        <v>168</v>
       </c>
       <c r="F33" t="n">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="G33" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H33" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -7654,13 +7670,13 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>1256</v>
+        <v>375</v>
       </c>
       <c r="M33" t="n">
-        <v>603</v>
+        <v>180</v>
       </c>
       <c r="N33" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="O33" s="6">
         <f>ROUND((E33*(1+(H33/100)*MAX(0,I33-100)/100)*(1+G33/100))*((D33+F33*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J33/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -7674,34 +7690,34 @@
       <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr">
         <is>
-          <t>Un regard, et ses ennemis se battent pour elle.</t>
+          <t>Sous l'éclipse, la bête l'emporte sur l'homme — et sa rage grandit avec ses blessures.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>kobold</t>
+          <t>sorciere_de_sang</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Kobold</t>
+          <t>Sorcière de sang</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>draconique</t>
+          <t>nocturne</t>
         </is>
       </c>
       <c r="D34" s="5" t="n">
-        <v>836</v>
+        <v>607</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>129</v>
+        <v>176</v>
       </c>
       <c r="F34" s="5" t="n">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="G34" s="5" t="n">
         <v>8</v>
@@ -7719,13 +7735,13 @@
         <v>0</v>
       </c>
       <c r="L34" s="5" t="n">
-        <v>425</v>
+        <v>388</v>
       </c>
       <c r="M34" s="5" t="n">
-        <v>204</v>
+        <v>186</v>
       </c>
       <c r="N34" s="5" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="O34" s="6">
         <f>ROUND((E34*(1+(H34/100)*MAX(0,I34-100)/100)*(1+G34/100))*((D34+F34*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J34/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -7739,34 +7755,34 @@
       <c r="R34" s="5" t="inlineStr"/>
       <c r="S34" s="5" t="inlineStr">
         <is>
-          <t>Petit, rusé, armé d'une lance trop grande pour lui.</t>
+          <t>Elle appelle ses familiers d'un murmure.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>cerbere</t>
+          <t>chevalier_de_l_eclipse</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Cerbère</t>
+          <t>Chevalier de l'éclipse</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>demoniaque</t>
+          <t>nocturne</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>858</v>
+        <v>713</v>
       </c>
       <c r="E35" t="n">
-        <v>133</v>
+        <v>86</v>
       </c>
       <c r="F35" t="n">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="G35" t="n">
         <v>8</v>
@@ -7784,10 +7800,10 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>438</v>
+        <v>400</v>
       </c>
       <c r="M35" t="n">
-        <v>210</v>
+        <v>192</v>
       </c>
       <c r="N35" t="n">
         <v>15</v>
@@ -7801,50 +7817,46 @@
         <v/>
       </c>
       <c r="Q35" t="inlineStr"/>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t>cerbere.png</t>
-        </is>
-      </c>
+      <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr">
         <is>
-          <t>Molosse à trois têtes gardant les portes de l'abîme.</t>
+          <t>Son armure noire rend chaque coup à celui qui l'a porté.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>dragonnet</t>
+          <t>vampire_noble</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Dragonnet</t>
+          <t>Vampire noble</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>draconique</t>
+          <t>nocturne</t>
         </is>
       </c>
       <c r="D36" s="5" t="n">
-        <v>515</v>
+        <v>814</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="F36" s="5" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="J36" s="5" t="n">
         <v>0</v>
@@ -7853,13 +7865,13 @@
         <v>0</v>
       </c>
       <c r="L36" s="5" t="n">
-        <v>438</v>
+        <v>412</v>
       </c>
       <c r="M36" s="5" t="n">
-        <v>210</v>
+        <v>198</v>
       </c>
       <c r="N36" s="5" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="O36" s="6">
         <f>ROUND((E36*(1+(H36/100)*MAX(0,I36-100)/100)*(1+G36/100))*((D36+F36*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J36/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -7873,43 +7885,43 @@
       <c r="R36" s="5" t="inlineStr"/>
       <c r="S36" s="5" t="inlineStr">
         <is>
-          <t>Un jeune dragon, vif et capricieux.</t>
+          <t>Il boit la vie de ses adversaires avec élégance.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>drake_de_braise</t>
+          <t>comtesse_ecarlate</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Drake de braise</t>
+          <t>Comtesse écarlate</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>draconique</t>
+          <t>nocturne</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>704</v>
+        <v>8910</v>
       </c>
       <c r="E37" t="n">
-        <v>204</v>
+        <v>344</v>
       </c>
       <c r="F37" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="G37" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I37" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -7918,13 +7930,13 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>450</v>
+        <v>1256</v>
       </c>
       <c r="M37" t="n">
-        <v>216</v>
+        <v>603</v>
       </c>
       <c r="N37" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="O37" s="6">
         <f>ROUND((E37*(1+(H37/100)*MAX(0,I37-100)/100)*(1+G37/100))*((D37+F37*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J37/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -7938,19 +7950,19 @@
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr">
         <is>
-          <t>Ses morsures laissent des brûlures qui couvent longtemps.</t>
+          <t>Un regard, et ses ennemis se battent pour elle.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>wyverne</t>
+          <t>kobold</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Wyverne</t>
+          <t>Kobold</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
@@ -7959,22 +7971,22 @@
         </is>
       </c>
       <c r="D38" s="5" t="n">
-        <v>541</v>
+        <v>836</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="F38" s="5" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G38" s="5" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="J38" s="5" t="n">
         <v>0</v>
@@ -7983,13 +7995,13 @@
         <v>0</v>
       </c>
       <c r="L38" s="5" t="n">
-        <v>462</v>
+        <v>425</v>
       </c>
       <c r="M38" s="5" t="n">
-        <v>222</v>
+        <v>204</v>
       </c>
       <c r="N38" s="5" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="O38" s="6">
         <f>ROUND((E38*(1+(H38/100)*MAX(0,I38-100)/100)*(1+G38/100))*((D38+F38*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J38/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -8003,19 +8015,19 @@
       <c r="R38" s="5" t="inlineStr"/>
       <c r="S38" s="5" t="inlineStr">
         <is>
-          <t>Elle fond sur sa proie et frappe deux fois avant qu'on la voie.</t>
+          <t>Petit, rusé, armé d'une lance trop grande pour lui.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>dragon_de_givre</t>
+          <t>dragonnet</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Dragon de givre</t>
+          <t>Dragonnet</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -8024,22 +8036,22 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>822</v>
+        <v>515</v>
       </c>
       <c r="E39" t="n">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="F39" t="n">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="G39" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="H39" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I39" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
@@ -8048,13 +8060,13 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>475</v>
+        <v>438</v>
       </c>
       <c r="M39" t="n">
-        <v>228</v>
+        <v>210</v>
       </c>
       <c r="N39" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="O39" s="6">
         <f>ROUND((E39*(1+(H39/100)*MAX(0,I39-100)/100)*(1+G39/100))*((D39+F39*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J39/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -8068,34 +8080,34 @@
       <c r="R39" t="inlineStr"/>
       <c r="S39" t="inlineStr">
         <is>
-          <t>Son souffle fige le sang dans les veines.</t>
+          <t>Un jeune dragon, vif et capricieux.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>succube</t>
+          <t>drake_de_braise</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Succube</t>
+          <t>Drake de braise</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>demoniaque</t>
+          <t>draconique</t>
         </is>
       </c>
       <c r="D40" s="5" t="n">
-        <v>748</v>
+        <v>704</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>220</v>
+        <v>204</v>
       </c>
       <c r="F40" s="5" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G40" s="5" t="n">
         <v>8</v>
@@ -8113,13 +8125,13 @@
         <v>0</v>
       </c>
       <c r="L40" s="5" t="n">
-        <v>488</v>
+        <v>450</v>
       </c>
       <c r="M40" s="5" t="n">
-        <v>234</v>
+        <v>216</v>
       </c>
       <c r="N40" s="5" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="O40" s="6">
         <f>ROUND((E40*(1+(H40/100)*MAX(0,I40-100)/100)*(1+G40/100))*((D40+F40*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J40/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -8130,26 +8142,22 @@
         <v/>
       </c>
       <c r="Q40" s="5" t="inlineStr"/>
-      <c r="R40" s="5" t="inlineStr">
-        <is>
-          <t>succube.png</t>
-        </is>
-      </c>
+      <c r="R40" s="5" t="inlineStr"/>
       <c r="S40" s="5" t="inlineStr">
         <is>
-          <t>Démone envoûtante qui draine la vie de ses proies.</t>
+          <t>Ses morsures laissent des brûlures qui couvent longtemps.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>gardien_draconique</t>
+          <t>wyverne</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Gardien draconique</t>
+          <t>Wyverne</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -8158,22 +8166,22 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>935</v>
+        <v>541</v>
       </c>
       <c r="E41" t="n">
-        <v>146</v>
+        <v>126</v>
       </c>
       <c r="F41" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="G41" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="H41" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I41" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="J41" t="n">
         <v>0</v>
@@ -8182,13 +8190,13 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>488</v>
+        <v>462</v>
       </c>
       <c r="M41" t="n">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="N41" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="O41" s="6">
         <f>ROUND((E41*(1+(H41/100)*MAX(0,I41-100)/100)*(1+G41/100))*((D41+F41*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J41/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -8202,19 +8210,19 @@
       <c r="R41" t="inlineStr"/>
       <c r="S41" t="inlineStr">
         <is>
-          <t>Une écaille-bouclier le protège avant qu'on puisse l'atteindre.</t>
+          <t>Elle fond sur sa proie et frappe deux fois avant qu'on la voie.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>dragon_ancien</t>
+          <t>dragon_de_givre</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Dragon ancien</t>
+          <t>Dragon de givre</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
@@ -8223,13 +8231,13 @@
         </is>
       </c>
       <c r="D42" s="5" t="n">
-        <v>19906</v>
+        <v>822</v>
       </c>
       <c r="E42" s="5" t="n">
-        <v>170</v>
+        <v>100</v>
       </c>
       <c r="F42" s="5" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="G42" s="5" t="n">
         <v>8</v>
@@ -8247,13 +8255,13 @@
         <v>0</v>
       </c>
       <c r="L42" s="5" t="n">
-        <v>1500</v>
+        <v>475</v>
       </c>
       <c r="M42" s="5" t="n">
-        <v>720</v>
+        <v>228</v>
       </c>
       <c r="N42" s="5" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="O42" s="6">
         <f>ROUND((E42*(1+(H42/100)*MAX(0,I42-100)/100)*(1+G42/100))*((D42+F42*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J42/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -8267,34 +8275,34 @@
       <c r="R42" s="5" t="inlineStr"/>
       <c r="S42" s="5" t="inlineStr">
         <is>
-          <t>Le maître des cimes. Blessé, il devient un brasier.</t>
+          <t>Son souffle fige le sang dans les veines.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>rejeton_du_neant</t>
+          <t>gardien_draconique</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Rejeton du néant</t>
+          <t>Gardien draconique</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>abyssal</t>
+          <t>draconique</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>968</v>
+        <v>935</v>
       </c>
       <c r="E43" t="n">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="F43" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G43" t="n">
         <v>8</v>
@@ -8312,13 +8320,13 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>506</v>
+        <v>488</v>
       </c>
       <c r="M43" t="n">
-        <v>243</v>
+        <v>234</v>
       </c>
       <c r="N43" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="O43" s="6">
         <f>ROUND((E43*(1+(H43/100)*MAX(0,I43-100)/100)*(1+G43/100))*((D43+F43*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J43/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -8332,43 +8340,43 @@
       <c r="R43" t="inlineStr"/>
       <c r="S43" t="inlineStr">
         <is>
-          <t>Une ombre qui a appris à marcher.</t>
+          <t>Une écaille-bouclier le protège avant qu'on puisse l'atteindre.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>oeil_errant</t>
+          <t>dragon_ancien</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Œil errant</t>
+          <t>Dragon ancien</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>abyssal</t>
+          <t>draconique</t>
         </is>
       </c>
       <c r="D44" s="5" t="n">
-        <v>601</v>
+        <v>19906</v>
       </c>
       <c r="E44" s="5" t="n">
-        <v>142</v>
+        <v>170</v>
       </c>
       <c r="F44" s="5" t="n">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="G44" s="5" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H44" s="5" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="I44" s="5" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="J44" s="5" t="n">
         <v>0</v>
@@ -8377,13 +8385,13 @@
         <v>0</v>
       </c>
       <c r="L44" s="5" t="n">
-        <v>525</v>
+        <v>1500</v>
       </c>
       <c r="M44" s="5" t="n">
-        <v>252</v>
+        <v>720</v>
       </c>
       <c r="N44" s="5" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O44" s="6">
         <f>ROUND((E44*(1+(H44/100)*MAX(0,I44-100)/100)*(1+G44/100))*((D44+F44*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J44/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -8397,34 +8405,34 @@
       <c r="R44" s="5" t="inlineStr"/>
       <c r="S44" s="5" t="inlineStr">
         <is>
-          <t>Il flotte, il observe, il ne cligne jamais.</t>
+          <t>Le maître des cimes. Blessé, il devient un brasier.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ange_dechu</t>
+          <t>rejeton_du_neant</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Ange déchu</t>
+          <t>Rejeton du néant</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>demoniaque</t>
+          <t>abyssal</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1034</v>
+        <v>968</v>
       </c>
       <c r="E45" t="n">
-        <v>163</v>
+        <v>153</v>
       </c>
       <c r="F45" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G45" t="n">
         <v>8</v>
@@ -8442,13 +8450,13 @@
         <v>0</v>
       </c>
       <c r="L45" t="n">
-        <v>544</v>
+        <v>506</v>
       </c>
       <c r="M45" t="n">
-        <v>261</v>
+        <v>243</v>
       </c>
       <c r="N45" t="n">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="O45" s="6">
         <f>ROUND((E45*(1+(H45/100)*MAX(0,I45-100)/100)*(1+G45/100))*((D45+F45*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J45/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -8459,26 +8467,22 @@
         <v/>
       </c>
       <c r="Q45" t="inlineStr"/>
-      <c r="R45" t="inlineStr">
-        <is>
-          <t>ange_dechu.png</t>
-        </is>
-      </c>
+      <c r="R45" t="inlineStr"/>
       <c r="S45" t="inlineStr">
         <is>
-          <t>Ancien séraphin banni ; sa lumière s'est muée en fureur.</t>
+          <t>Une ombre qui a appris à marcher.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>devoreur</t>
+          <t>oeil_errant</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Dévoreur</t>
+          <t>Œil errant</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
@@ -8487,22 +8491,22 @@
         </is>
       </c>
       <c r="D46" s="5" t="n">
-        <v>827</v>
+        <v>601</v>
       </c>
       <c r="E46" s="5" t="n">
-        <v>245</v>
+        <v>142</v>
       </c>
       <c r="F46" s="5" t="n">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I46" s="5" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="J46" s="5" t="n">
         <v>0</v>
@@ -8511,13 +8515,13 @@
         <v>0</v>
       </c>
       <c r="L46" s="5" t="n">
-        <v>544</v>
+        <v>525</v>
       </c>
       <c r="M46" s="5" t="n">
-        <v>261</v>
+        <v>252</v>
       </c>
       <c r="N46" s="5" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="O46" s="6">
         <f>ROUND((E46*(1+(H46/100)*MAX(0,I46-100)/100)*(1+G46/100))*((D46+F46*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J46/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -8531,19 +8535,19 @@
       <c r="R46" s="5" t="inlineStr"/>
       <c r="S46" s="5" t="inlineStr">
         <is>
-          <t>Il se nourrit de tout ce qu'il touche — et se referme sur ses plaies.</t>
+          <t>Il flotte, il observe, il ne cligne jamais.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>heraut_du_vide</t>
+          <t>devoreur</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Héraut du vide</t>
+          <t>Dévoreur</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -8552,13 +8556,13 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1067</v>
+        <v>827</v>
       </c>
       <c r="E47" t="n">
-        <v>168</v>
+        <v>245</v>
       </c>
       <c r="F47" t="n">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="G47" t="n">
         <v>8</v>
@@ -8576,13 +8580,13 @@
         <v>0</v>
       </c>
       <c r="L47" t="n">
-        <v>562</v>
+        <v>544</v>
       </c>
       <c r="M47" t="n">
-        <v>270</v>
+        <v>261</v>
       </c>
       <c r="N47" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="O47" s="6">
         <f>ROUND((E47*(1+(H47/100)*MAX(0,I47-100)/100)*(1+G47/100))*((D47+F47*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J47/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -8596,19 +8600,19 @@
       <c r="R47" t="inlineStr"/>
       <c r="S47" t="inlineStr">
         <is>
-          <t>Il ouvre des failles d'où rampent d'autres créatures.</t>
+          <t>Il se nourrit de tout ce qu'il touche — et se referme sur ses plaies.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>kraken_astral</t>
+          <t>heraut_du_vide</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>Kraken astral</t>
+          <t>Héraut du vide</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
@@ -8617,13 +8621,13 @@
         </is>
       </c>
       <c r="D48" s="5" t="n">
-        <v>990</v>
+        <v>1067</v>
       </c>
       <c r="E48" s="5" t="n">
-        <v>121</v>
+        <v>168</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="G48" s="5" t="n">
         <v>8</v>
@@ -8641,13 +8645,13 @@
         <v>0</v>
       </c>
       <c r="L48" s="5" t="n">
-        <v>581</v>
+        <v>562</v>
       </c>
       <c r="M48" s="5" t="n">
-        <v>279</v>
+        <v>270</v>
       </c>
       <c r="N48" s="5" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="O48" s="6">
         <f>ROUND((E48*(1+(H48/100)*MAX(0,I48-100)/100)*(1+G48/100))*((D48+F48*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J48/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -8661,19 +8665,19 @@
       <c r="R48" s="5" t="inlineStr"/>
       <c r="S48" s="5" t="inlineStr">
         <is>
-          <t>Ses tentacules frappent de toutes parts et engourdissent.</t>
+          <t>Il ouvre des failles d'où rampent d'autres créatures.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>seraphin_brise</t>
+          <t>kraken_astral</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Séraphin brisé</t>
+          <t>Kraken astral</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -8682,13 +8686,13 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>906</v>
+        <v>990</v>
       </c>
       <c r="E49" t="n">
-        <v>270</v>
+        <v>121</v>
       </c>
       <c r="F49" t="n">
-        <v>23</v>
+        <v>60</v>
       </c>
       <c r="G49" t="n">
         <v>8</v>
@@ -8706,13 +8710,13 @@
         <v>0</v>
       </c>
       <c r="L49" t="n">
-        <v>600</v>
+        <v>581</v>
       </c>
       <c r="M49" t="n">
-        <v>288</v>
+        <v>279</v>
       </c>
       <c r="N49" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="O49" s="6">
         <f>ROUND((E49*(1+(H49/100)*MAX(0,I49-100)/100)*(1+G49/100))*((D49+F49*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J49/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -8726,34 +8730,34 @@
       <c r="R49" t="inlineStr"/>
       <c r="S49" t="inlineStr">
         <is>
-          <t>Un ange tombé dans la faille ; il refuse de mourir.</t>
+          <t>Ses tentacules frappent de toutes parts et engourdissent.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>archidemon</t>
+          <t>seraphin_brise</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>Archidémon</t>
+          <t>Séraphin brisé</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>demoniaque</t>
+          <t>abyssal</t>
         </is>
       </c>
       <c r="D50" s="5" t="n">
-        <v>18533</v>
+        <v>906</v>
       </c>
       <c r="E50" s="5" t="n">
-        <v>381</v>
+        <v>270</v>
       </c>
       <c r="F50" s="5" t="n">
-        <v>62</v>
+        <v>23</v>
       </c>
       <c r="G50" s="5" t="n">
         <v>8</v>
@@ -8771,13 +8775,13 @@
         <v>0</v>
       </c>
       <c r="L50" s="5" t="n">
-        <v>1819</v>
+        <v>600</v>
       </c>
       <c r="M50" s="5" t="n">
-        <v>873</v>
+        <v>288</v>
       </c>
       <c r="N50" s="5" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="O50" s="6">
         <f>ROUND((E50*(1+(H50/100)*MAX(0,I50-100)/100)*(1+G50/100))*((D50+F50*'⚙️ Calibrage'!$B$9)/MAX(0.01,1-J50/100))/'⚙️ Calibrage'!$B$10,0)</f>
@@ -8788,14 +8792,10 @@
         <v/>
       </c>
       <c r="Q50" s="5" t="inlineStr"/>
-      <c r="R50" s="5" t="inlineStr">
-        <is>
-          <t>archidemon.png</t>
-        </is>
-      </c>
+      <c r="R50" s="5" t="inlineStr"/>
       <c r="S50" s="5" t="inlineStr">
         <is>
-          <t>Seigneur des enfers, apogée de la corruption du Berceau.</t>
+          <t>Un ange tombé dans la faille ; il refuse de mourir.</t>
         </is>
       </c>
     </row>
@@ -8819,7 +8819,7 @@
         <v>21186</v>
       </c>
       <c r="E51" t="n">
-        <v>373</v>
+        <v>280</v>
       </c>
       <c r="F51" t="n">
         <v>48</v>
@@ -10967,7 +10967,7 @@
         </is>
       </c>
       <c r="E2" s="5" t="n">
-        <v>1000</v>
+        <v>550</v>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
@@ -11012,7 +11012,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>1500</v>
+        <v>900</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -11057,7 +11057,7 @@
         </is>
       </c>
       <c r="E4" s="5" t="n">
-        <v>2600</v>
+        <v>1200</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
@@ -11116,7 +11116,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>oui</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -11161,7 +11161,7 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>oui</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -11206,7 +11206,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>oui</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">

</xml_diff>

<commit_message>
feat(combat): combats contre plusieurs ennemis et passifs des 27 pièces C → S
Le moteur gère désormais un groupe d'ennemis (tour solo, meutes) :
chacun a sa jauge, ses capacités, son escalade et sa provocation ; les
joueurs se concentrent sur le plus abîmé ; l'AOE de l'arbre touche les
voisins de la cible. Un seul ennemi = le même combat qu'avant.

Les 27 pièces des zones C → S reçoivent leur passif, avec les
ajustements de l'auteur (Sève plafonnée, Mousse vivace, Festin 25 %,
Pacte de sang avec érosion, Braise persistante, Souffle ancestral en
exécution, Dévoration, Néant dévorant).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sakura_content.xlsx
+++ b/docs/sakura_content.xlsx
@@ -511,7 +511,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 2026-10-27 07:50 UTC</t>
+          <t>Généré le 2026-10-27 08:03 UTC</t>
         </is>
       </c>
     </row>
@@ -1753,7 +1753,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Festin de chair — Chaque ennemi vaincu te rend 25 % de tes PV max.</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr"/>
@@ -1829,7 +1829,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Embuscade — +25 % de dégâts contre un ennemi qui n'a pas encore agi.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -1981,7 +1981,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Soif écarlate — Tes coups critiques te soignent de 20 % des dégâts infligés.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -2437,7 +2437,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Miroir d'éclipse — 15 % des dégâts que tu reçois sont renvoyés à l'attaquant.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Morsure du givre — 15 % de chance de geler l'ennemi qui te frappe : il perd sa prochaine action (pas les boss).</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr"/>
@@ -2665,7 +2665,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pacte de sang — À court de mana, tes compétences se paient en PV : 5 % de tes PV max, et l'érosion réduit tes PV max de 5 % pour le reste du combat.</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr"/>
@@ -2817,7 +2817,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Échos du vide — Toutes les 8 actions, un écho frappe la cible (50 % de ton attaque, sans défense) et absorbe le prochain coup que tu reçois.</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr"/>
@@ -3045,7 +3045,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Piqué — Ta première attaque frappe 3 fois, à 60 % chacune.</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
@@ -3121,7 +3121,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ramure bienveillante — Tout le groupe reçoit 15 % de soins en plus (une seule ramure par groupe).</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr"/>
@@ -3425,7 +3425,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rage lunaire — Sous 50 % de PV : +15 % d'attaque et de vitesse.</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr"/>
@@ -3653,7 +3653,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Coup de patte brisant — Chaque coup réduit la défense de l'ennemi de 3 % pour le combat (max −15 %, non cumulable).</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
@@ -3729,7 +3729,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Vol nocturne — +5 % d'esquive tant que tu es au-dessus de 50 % de tes PV.</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr"/>
@@ -3805,7 +3805,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Grâce brisée — Le premier allié qui tombe se relève avec 30 % de ses PV (une fois par combat).</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
@@ -3881,7 +3881,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Valse sanglante — Après chaque esquive, ton coup suivant est un critique qui fait saigner (10 % des dégâts à chaque action de l'ennemi, 3 actions, jusqu'à 3 fois).</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr"/>
@@ -4261,7 +4261,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Instinct de meute — +3 % de dégâts par allié encore debout (max +9 %).</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
@@ -4337,7 +4337,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Braise persistante — Tes critiques enflamment l'ennemi : −20 % d'attaque pendant 2 actions (non cumulable) et 10 % des dégâts du coup à chacune de ses 2 actions suivantes (cumulable).</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr"/>
@@ -4413,7 +4413,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Mousse vivace — La première fois que tu passes sous 30 % de PV, tu récupères 10 % de tes PV max à chacune de tes 7 actions suivantes.</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
@@ -4489,7 +4489,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Néant dévorant — Un coup sur deux ignore 50 % de la défense ennemie.</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr"/>
@@ -4565,7 +4565,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Souffle ancestral — Exécute la cible de ton attaque si elle passe sous 20 % de ses PV (les boss y sont immunisés).</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
@@ -4641,7 +4641,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Souffle juvénile — Toutes les 5 attaques, des flammes frappent tous les ennemis (30 % de ton attaque, sans défense).</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr"/>
@@ -4717,7 +4717,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Réserve abyssale — Tes compétences coûtent 20 % de mana en moins.</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
@@ -4869,7 +4869,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Dévoration — Quand un allié meurt, tu gagnes 10 % de son attaque, de sa défense et de ses PV max pour le reste du combat.</t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
@@ -5021,7 +5021,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Œil de la tempête — Ta première action frappe TOUS les ennemis, avec 50 % de chance d'étourdir chacun (pas les boss).</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
@@ -5097,7 +5097,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Serment du gardien — Tant que tu provoques : −20 % de dégâts reçus pour toi, −10 % pour tes alliés.</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr"/>
@@ -5173,7 +5173,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Étreinte astrale — Tes coups ralentissent l'ennemi de 5 % (max −25 %, non cumulable).</t>
         </is>
       </c>
       <c r="G49" t="inlineStr"/>
@@ -5249,7 +5249,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sève vénéneuse — Tes coups empoisonnent l'ennemi : 1 % de ses PV max à chacune de ses actions pendant 3 actions, au plus 25 % de ton attaque (non cumulable).</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr"/>
@@ -5325,7 +5325,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Regard du vide — L'ennemi ne peut pas esquiver tes coups.</t>
         </is>
       </c>
       <c r="G51" t="inlineStr"/>

</xml_diff>

<commit_message>
feat(tuto): tutoriel RP de Hana, panneau du salon tutoriel, 3 potions 100 % PV
- /tuto (salon tutoriel + salons de commandes) et panneau permanent :
  suivre le tutoriel ou le passer et commencer l'aventure.
- 10 étapes RP avec actions vérifiées (/daily, /stats, premier combat,
  voyante), progression gardée (player_tutorials, migration c4e8a2d6f913).
- Fin : rôle Rang F et 3 Potions du Grand Cerisier (100 % des PV), une fois.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sakura_content.xlsx
+++ b/docs/sakura_content.xlsx
@@ -22,7 +22,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'🎽 Équipements'!$A$1:$T$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'👹 Mobs'!$A$1:$S$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'🧪 Consommables'!$A$1:$H$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'🧪 Consommables'!$A$1:$H$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'⚗️ Alchimie'!$A$1:$F$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'📦 Ressources'!$A$1:$H$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'🏪 Shop'!$A$1:$I$34</definedName>
@@ -511,7 +511,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 2026-10-27 14:47 UTC</t>
+          <t>Généré le 2026-10-31 18:41 UTC</t>
         </is>
       </c>
     </row>
@@ -8882,7 +8882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -8976,17 +8976,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>potion_soin_superieure</t>
+          <t>potion_soin_totale</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Potion de soin supérieure</t>
+          <t>Potion du Grand Cerisier</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>common</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -8995,7 +8995,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -9005,19 +9005,19 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Rend 35 % des PV max (sans dépasser le maximum).</t>
+          <t>Rend 100 % des PV max. Offerte par Hana à la fin du tutoriel (/tuto).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>potion_mana</t>
+          <t>potion_soin_superieure</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Potion de mana</t>
+          <t>Potion de soin supérieure</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -9027,11 +9027,11 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>mana_percent</t>
+          <t>heal_percent</t>
         </is>
       </c>
       <c r="E4" s="5" t="n">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>0</v>
@@ -9041,19 +9041,19 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Rend 50 % du mana max (sans dépasser le maximum).</t>
+          <t>Rend 35 % des PV max (sans dépasser le maximum).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>elixir_recuperation</t>
+          <t>potion_mana</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Élixir de récupération</t>
+          <t>Potion de mana</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -9063,11 +9063,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>elixir</t>
+          <t>mana_percent</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>50</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -9077,19 +9077,19 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Pendant 1 h, tes PV et ton mana remontent 3 fois plus vite hors combat. Le reboire renouvelle sa durée.</t>
+          <t>Rend 50 % du mana max (sans dépasser le maximum).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>elixir_force</t>
+          <t>elixir_recuperation</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Élixir de force</t>
+          <t>Élixir de récupération</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -9103,7 +9103,7 @@
         </is>
       </c>
       <c r="E6" s="5" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>0</v>
@@ -9113,19 +9113,19 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>+10 % d'attaque pendant 1 h, en combat de zone et au world boss (pas en épreuve ni en défi). Le reboire renouvelle sa durée.</t>
+          <t>Pendant 1 h, tes PV et ton mana remontent 3 fois plus vite hors combat. Le reboire renouvelle sa durée.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>elixir_garde</t>
+          <t>elixir_force</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Élixir de garde</t>
+          <t>Élixir de force</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -9149,19 +9149,19 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>+10 % de défense pendant 1 h, en combat de zone et au world boss (pas en épreuve ni en défi). Le reboire renouvelle sa durée.</t>
+          <t>+10 % d'attaque pendant 1 h, en combat de zone et au world boss (pas en épreuve ni en défi). Le reboire renouvelle sa durée.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>elixir_vitalite</t>
+          <t>elixir_garde</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Élixir de vitalité</t>
+          <t>Élixir de garde</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -9185,19 +9185,19 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>+10 % de PV max pendant 1 h, en combat de zone et au world boss (pas en épreuve ni en défi). Le reboire renouvelle sa durée.</t>
+          <t>+10 % de défense pendant 1 h, en combat de zone et au world boss (pas en épreuve ni en défi). Le reboire renouvelle sa durée.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>grande_potion_soin</t>
+          <t>elixir_vitalite</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Grande potion de soin</t>
+          <t>Élixir de vitalité</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -9207,11 +9207,11 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>heal_percent</t>
+          <t>elixir</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
@@ -9221,19 +9221,19 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Rend 60 % des PV max (sans dépasser le maximum).</t>
+          <t>+10 % de PV max pendant 1 h, en combat de zone et au world boss (pas en épreuve ni en défi). Le reboire renouvelle sa durée.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>grande_potion_mana</t>
+          <t>grande_potion_soin</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Grande potion de mana</t>
+          <t>Grande potion de soin</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -9243,11 +9243,11 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>mana_percent</t>
+          <t>heal_percent</t>
         </is>
       </c>
       <c r="E10" s="5" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0</v>
@@ -9257,19 +9257,19 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Rend tout le mana.</t>
+          <t>Rend 60 % des PV max (sans dépasser le maximum).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>elixir_recuperation_sup</t>
+          <t>grande_potion_mana</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Élixir de récupération supérieur</t>
+          <t>Grande potion de mana</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -9279,11 +9279,11 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>elixir</t>
+          <t>mana_percent</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
@@ -9293,19 +9293,19 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Pendant 1 h, tes PV et ton mana remontent 5 fois plus vite hors combat. Le reboire renouvelle sa durée ; un élixir plus faible du même type ne le remplace pas.</t>
+          <t>Rend tout le mana.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>elixir_force_sup</t>
+          <t>elixir_recuperation_sup</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Élixir de force supérieur</t>
+          <t>Élixir de récupération supérieur</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -9319,7 +9319,7 @@
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>0</v>
@@ -9329,19 +9329,19 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>+20 % d'attaque pendant 1 h, en combat de zone et au world boss (pas en épreuve ni en défi). Le reboire renouvelle sa durée ; un élixir plus faible du même type ne le remplace pas.</t>
+          <t>Pendant 1 h, tes PV et ton mana remontent 5 fois plus vite hors combat. Le reboire renouvelle sa durée ; un élixir plus faible du même type ne le remplace pas.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>elixir_garde_sup</t>
+          <t>elixir_force_sup</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Élixir de garde supérieur</t>
+          <t>Élixir de force supérieur</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -9365,19 +9365,19 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>+20 % de défense pendant 1 h, en combat de zone et au world boss (pas en épreuve ni en défi). Le reboire renouvelle sa durée ; un élixir plus faible du même type ne le remplace pas.</t>
+          <t>+20 % d'attaque pendant 1 h, en combat de zone et au world boss (pas en épreuve ni en défi). Le reboire renouvelle sa durée ; un élixir plus faible du même type ne le remplace pas.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>elixir_vitalite_sup</t>
+          <t>elixir_garde_sup</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Élixir de vitalité supérieur</t>
+          <t>Élixir de garde supérieur</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -9401,19 +9401,19 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>+20 % de PV max pendant 1 h, en combat de zone et au world boss (pas en épreuve ni en défi). Le reboire renouvelle sa durée ; un élixir plus faible du même type ne le remplace pas.</t>
+          <t>+20 % de défense pendant 1 h, en combat de zone et au world boss (pas en épreuve ni en défi). Le reboire renouvelle sa durée ; un élixir plus faible du même type ne le remplace pas.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>cor_chasse_f</t>
+          <t>elixir_vitalite_sup</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Cor de chasse de la Clairière</t>
+          <t>Élixir de vitalité supérieur</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -9423,10 +9423,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>summon_elite</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
+          <t>elixir</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>20</v>
+      </c>
       <c r="F15" t="n">
         <v>0</v>
       </c>
@@ -9435,19 +9437,19 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Fait apparaître l'élite de la Clairière sinistre (rang F) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
+          <t>+20 % de PV max pendant 1 h, en combat de zone et au world boss (pas en épreuve ni en défi). Le reboire renouvelle sa durée ; un élixir plus faible du même type ne le remplace pas.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>cor_chasse_e</t>
+          <t>cor_chasse_f</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Cor de chasse du Cimetière</t>
+          <t>Cor de chasse de la Clairière</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -9469,19 +9471,19 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Fait apparaître l'élite du Cimetière abandonné (rang E) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
+          <t>Fait apparaître l'élite de la Clairière sinistre (rang F) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>cor_chasse_d</t>
+          <t>cor_chasse_e</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Cor de chasse du Berceau</t>
+          <t>Cor de chasse du Cimetière</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -9503,19 +9505,19 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Fait apparaître l'élite du Berceau cataclysmique (rang D) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
+          <t>Fait apparaître l'élite du Cimetière abandonné (rang E) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>cor_chasse_c</t>
+          <t>cor_chasse_d</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Cor de chasse du Sanctuaire</t>
+          <t>Cor de chasse du Berceau</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -9537,19 +9539,19 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Fait apparaître l'élite du Sanctuaire primordial (rang C) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
+          <t>Fait apparaître l'élite du Berceau cataclysmique (rang D) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>cor_chasse_b</t>
+          <t>cor_chasse_c</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Cor de chasse de l'Éclipse</t>
+          <t>Cor de chasse du Sanctuaire</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -9571,19 +9573,19 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Fait apparaître l'élite de l'Éclipse éternelle (rang B) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
+          <t>Fait apparaître l'élite du Sanctuaire primordial (rang C) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>cor_chasse_a</t>
+          <t>cor_chasse_b</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Cor de chasse des Cimes</t>
+          <t>Cor de chasse de l'Éclipse</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -9605,19 +9607,19 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Fait apparaître l'élite des Cimes des Wyrms (rang A) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
+          <t>Fait apparaître l'élite de l'Éclipse éternelle (rang B) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>sceau_souffle_e</t>
+          <t>cor_chasse_a</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Sceau du second souffle (rang E)</t>
+          <t>Cor de chasse des Cimes</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -9627,7 +9629,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>trial_retry</t>
+          <t>summon_elite</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
@@ -9639,19 +9641,19 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Efface l'attente après un échec à l'épreuve du rang E : tu peux la retenter tout de suite.</t>
+          <t>Fait apparaître l'élite des Cimes des Wyrms (rang A) dans le salon de la zone, à la suite du combat en cours. Il faut avoir accès à la zone ; 1 h d'attente entre deux cors, une seule élite invoquée par zone à la fois.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>sceau_souffle_d</t>
+          <t>sceau_souffle_e</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Sceau du second souffle (rang D)</t>
+          <t>Sceau du second souffle (rang E)</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -9673,19 +9675,19 @@
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>Efface l'attente après un échec à l'épreuve du rang D : tu peux la retenter tout de suite.</t>
+          <t>Efface l'attente après un échec à l'épreuve du rang E : tu peux la retenter tout de suite.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>sceau_souffle_c</t>
+          <t>sceau_souffle_d</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Sceau du second souffle (rang C)</t>
+          <t>Sceau du second souffle (rang D)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -9707,19 +9709,19 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Efface l'attente après un échec à l'épreuve du rang C : tu peux la retenter tout de suite.</t>
+          <t>Efface l'attente après un échec à l'épreuve du rang D : tu peux la retenter tout de suite.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>sceau_souffle_b</t>
+          <t>sceau_souffle_c</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Sceau du second souffle (rang B)</t>
+          <t>Sceau du second souffle (rang C)</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
@@ -9741,19 +9743,19 @@
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>Efface l'attente après un échec à l'épreuve du rang B : tu peux la retenter tout de suite.</t>
+          <t>Efface l'attente après un échec à l'épreuve du rang C : tu peux la retenter tout de suite.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>sceau_souffle_a</t>
+          <t>sceau_souffle_b</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Sceau du second souffle (rang A)</t>
+          <t>Sceau du second souffle (rang B)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -9775,19 +9777,19 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Efface l'attente après un échec à l'épreuve du rang A : tu peux la retenter tout de suite.</t>
+          <t>Efface l'attente après un échec à l'épreuve du rang B : tu peux la retenter tout de suite.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>sceau_souffle_s</t>
+          <t>sceau_souffle_a</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Sceau du second souffle (rang S)</t>
+          <t>Sceau du second souffle (rang A)</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
@@ -9809,19 +9811,19 @@
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>Efface l'attente après un échec à l'épreuve du rang S : tu peux la retenter tout de suite.</t>
+          <t>Efface l'attente après un échec à l'épreuve du rang A : tu peux la retenter tout de suite.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>sceau_souffle_ss</t>
+          <t>sceau_souffle_s</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Sceau du second souffle (rang SS)</t>
+          <t>Sceau du second souffle (rang S)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -9843,19 +9845,19 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Efface l'attente après un échec à l'épreuve du rang SS : tu peux la retenter tout de suite.</t>
+          <t>Efface l'attente après un échec à l'épreuve du rang S : tu peux la retenter tout de suite.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>sceau_souffle_sss</t>
+          <t>sceau_souffle_ss</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Sceau du second souffle (rang SSS)</t>
+          <t>Sceau du second souffle (rang SS)</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
@@ -9877,19 +9879,19 @@
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>Efface l'attente après un échec à l'épreuve du rang SSS : tu peux la retenter tout de suite.</t>
+          <t>Efface l'attente après un échec à l'épreuve du rang SS : tu peux la retenter tout de suite.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>parchemin_oubli</t>
+          <t>sceau_souffle_sss</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Parchemin d'oubli</t>
+          <t>Sceau du second souffle (rang SSS)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -9899,7 +9901,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>respec_stats</t>
+          <t>trial_retry</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
@@ -9911,19 +9913,19 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Reprend TOUS tes points de stats (attaque, défense, PV) : replace-les ensuite avec /stats.</t>
+          <t>Efface l'attente après un échec à l'épreuve du rang SSS : tu peux la retenter tout de suite.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>jeton_arbre</t>
+          <t>parchemin_oubli</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Jeton de réinitialisation d'arbre</t>
+          <t>Parchemin d'oubli</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
@@ -9933,7 +9935,7 @@
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>reset_tree</t>
+          <t>respec_stats</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr"/>
@@ -9945,19 +9947,19 @@
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>Réinitialise ton arbre de compétences EN PLUS du reset gratuit de la semaine (à garder pour quand il est déjà pris).</t>
+          <t>Reprend TOUS tes points de stats (attaque, défense, PV) : replace-les ensuite avec /stats.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>sablier_fidelite</t>
+          <t>jeton_arbre</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sablier de fidélité</t>
+          <t>Jeton de réinitialisation d'arbre</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -9967,7 +9969,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>daily_guard</t>
+          <t>reset_tree</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
@@ -9979,12 +9981,46 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
+          <t>Réinitialise ton arbre de compétences EN PLUS du reset gratuit de la semaine (à garder pour quand il est déjà pris).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>sablier_fidelite</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Sablier de fidélité</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>daily_guard</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr"/>
+      <c r="F32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
           <t>Le premier jour de /daily manqué, ta série n'est pas divisée par deux. Il agit tout seul ; un seul à la fois.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H31"/>
+  <autoFilter ref="A1:H32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>